<commit_message>
Add one more row in title excel file
</commit_message>
<xml_diff>
--- a/inst/extdata/sample_titles2.xlsx
+++ b/inst/extdata/sample_titles2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u066227\TFootr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97278FCE-AAB9-4248-BE15-489D79AF8D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77498BA8-4F73-4E04-BA1A-DCCCE046BBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{30221CC8-E0E7-4D3A-9A2D-9EE88E0E375F}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="126">
   <si>
     <t>Pgmname</t>
   </si>
@@ -410,6 +410,36 @@
   <si>
     <t>Test Subtitle to Show Example</t>
   </si>
+  <si>
+    <t>Figure</t>
+  </si>
+  <si>
+    <t>ggplot-example1.rmd</t>
+  </si>
+  <si>
+    <t>mtcars</t>
+  </si>
+  <si>
+    <t>mtcars Population</t>
+  </si>
+  <si>
+    <t>Figure 1.2</t>
+  </si>
+  <si>
+    <t>Sample Figure with mtcars Data</t>
+  </si>
+  <si>
+    <t>Test Subtitle1</t>
+  </si>
+  <si>
+    <t>Sample footnote 1: This is an example to show how to use tfootr package for processing footnotes.</t>
+  </si>
+  <si>
+    <t>Sample footnote 2: The second line of footnote example.</t>
+  </si>
+  <si>
+    <t>Third footnote example.</t>
+  </si>
 </sst>
 </file>
 
@@ -418,8 +448,8 @@
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_-&quot;€&quot;* #,##0_-;\-&quot;€&quot;* #,##0_-;_-&quot;€&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;€&quot;* #,##0_-;\-&quot;€&quot;* #,##0_-;_-&quot;€&quot;* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="43">
     <font>
@@ -1171,17 +1201,17 @@
     <xf numFmtId="0" fontId="25" fillId="33" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="34" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1275,29 +1305,25 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="39" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="39" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="39" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="39" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1308,59 +1334,49 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="126">
     <cellStyle name="20% - Accent1 2" xfId="1" xr:uid="{A1F0AB5F-07D9-4BF8-A4A9-AF96D9E333E5}"/>
@@ -1884,388 +1900,388 @@
   <dimension ref="A1:T11"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="26.6328125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" style="13" customWidth="1"/>
-    <col min="4" max="5" width="14.7265625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.54296875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" style="14" customWidth="1"/>
-    <col min="8" max="8" width="51.54296875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="27.453125" style="12" customWidth="1"/>
-    <col min="10" max="10" width="17.26953125" style="12" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" style="12" customWidth="1"/>
-    <col min="12" max="12" width="9.1796875" style="12"/>
-    <col min="13" max="13" width="40" style="15" customWidth="1"/>
-    <col min="14" max="14" width="39.26953125" style="15" customWidth="1"/>
-    <col min="15" max="15" width="37.1796875" style="15" customWidth="1"/>
-    <col min="16" max="16" width="30.54296875" style="12" customWidth="1"/>
-    <col min="17" max="17" width="27.1796875" style="12" customWidth="1"/>
-    <col min="18" max="18" width="126" style="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.1796875" style="12"/>
+    <col min="1" max="1" width="26.6328125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" style="9" customWidth="1"/>
+    <col min="4" max="5" width="14.7265625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="24.54296875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="51.54296875" style="11" customWidth="1"/>
+    <col min="9" max="9" width="27.453125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="9.1796875" style="8"/>
+    <col min="13" max="13" width="40" style="11" customWidth="1"/>
+    <col min="14" max="14" width="39.26953125" style="11" customWidth="1"/>
+    <col min="15" max="15" width="37.1796875" style="11" customWidth="1"/>
+    <col min="16" max="16" width="30.54296875" style="8" customWidth="1"/>
+    <col min="17" max="17" width="27.1796875" style="8" customWidth="1"/>
+    <col min="18" max="18" width="126" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.1796875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="8" customFormat="1" ht="13">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:20" s="4" customFormat="1" ht="13">
+      <c r="A1" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="S1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="T1" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="35" customFormat="1" ht="25.5">
-      <c r="A2" s="33" t="s">
+    <row r="2" spans="1:20" s="27" customFormat="1" ht="25.5">
+      <c r="A2" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="34" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11" t="s">
+      <c r="D2" s="7"/>
+      <c r="E2" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="11"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="10" t="str">
+      <c r="I2" s="7"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="6" t="str">
         <f>[1]Footnotes!A1</f>
         <v>Footnotes</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
     </row>
     <row r="3" spans="1:20" ht="25">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="N3" s="15" t="s">
+      <c r="N3" s="11" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="27">
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="M4" s="36" t="s">
+      <c r="M4" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="N4" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="O4" s="36" t="s">
+      <c r="O4" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="P4" s="36" t="s">
+      <c r="P4" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="Q4" s="12" t="s">
+      <c r="Q4" s="8" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="13.5">
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M5" s="36" t="s">
+      <c r="M5" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="N5" s="36" t="s">
+      <c r="N5" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="O5" s="36" t="s">
+      <c r="O5" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="P5" s="36" t="s">
+      <c r="P5" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="Q5" s="12" t="s">
+      <c r="Q5" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="R5" s="12" t="s">
+      <c r="R5" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="13.5">
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="M6" s="36" t="s">
+      <c r="M6" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="N6" s="15" t="s">
+      <c r="N6" s="11" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="13.5">
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="11" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="13.5">
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="M8" s="36" t="s">
+      <c r="M8" s="28" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:20" ht="25">
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M9" s="36" t="s">
+      <c r="M9" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="N9" s="15" t="s">
+      <c r="N9" s="11" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="13.5">
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="M10" s="36" t="s">
+      <c r="M10" s="28" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="13.5">
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="M11" s="36" t="s">
+      <c r="M11" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="N11" s="15" t="s">
+      <c r="N11" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="O11" s="36" t="s">
+      <c r="O11" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="P11" s="36" t="s">
+      <c r="P11" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="Q11" s="12" t="s">
+      <c r="Q11" s="8" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2280,392 +2296,424 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57BBBF2B-056A-4DC3-A47F-4EB17BAEC258}">
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="26.6328125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" style="13" customWidth="1"/>
-    <col min="4" max="5" width="14.7265625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.54296875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" style="14" customWidth="1"/>
-    <col min="8" max="8" width="51.54296875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="27.453125" style="12" customWidth="1"/>
-    <col min="10" max="10" width="17.26953125" style="12" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" style="12" customWidth="1"/>
-    <col min="12" max="12" width="9.1796875" style="12"/>
-    <col min="13" max="13" width="40" style="15" customWidth="1"/>
-    <col min="14" max="14" width="39.26953125" style="15" customWidth="1"/>
-    <col min="15" max="15" width="37.1796875" style="15" customWidth="1"/>
-    <col min="16" max="16" width="30.54296875" style="12" customWidth="1"/>
-    <col min="17" max="17" width="27.1796875" style="12" customWidth="1"/>
-    <col min="18" max="18" width="126" style="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.1796875" style="12"/>
+    <col min="1" max="1" width="26.6328125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" style="9" customWidth="1"/>
+    <col min="4" max="5" width="14.7265625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="24.54296875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="51.54296875" style="11" customWidth="1"/>
+    <col min="9" max="9" width="27.453125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="9.1796875" style="8"/>
+    <col min="13" max="13" width="40" style="11" customWidth="1"/>
+    <col min="14" max="14" width="39.26953125" style="11" customWidth="1"/>
+    <col min="15" max="15" width="37.1796875" style="11" customWidth="1"/>
+    <col min="16" max="16" width="30.54296875" style="8" customWidth="1"/>
+    <col min="17" max="17" width="27.1796875" style="8" customWidth="1"/>
+    <col min="18" max="18" width="28.26953125" style="8" customWidth="1"/>
+    <col min="19" max="16384" width="9.1796875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="8" customFormat="1" ht="13">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:20" s="4" customFormat="1" ht="13">
+      <c r="A1" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="S1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="T1" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="35" customFormat="1" ht="25.5">
-      <c r="A2" s="33" t="s">
+    <row r="2" spans="1:20" s="27" customFormat="1" ht="25.5">
+      <c r="A2" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="34" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11" t="s">
+      <c r="D2" s="7"/>
+      <c r="E2" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="11"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="10" t="str">
+      <c r="I2" s="7"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="6" t="str">
         <f>[1]Footnotes!A1</f>
         <v>Footnotes</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
     </row>
     <row r="3" spans="1:20" ht="25">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="N3" s="15" t="s">
+      <c r="N3" s="11" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="27">
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="M4" s="36" t="s">
+      <c r="M4" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="N4" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="O4" s="36" t="s">
+      <c r="O4" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="P4" s="36" t="s">
+      <c r="P4" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="Q4" s="12" t="s">
+      <c r="Q4" s="8" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="13.5">
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M5" s="36" t="s">
+      <c r="M5" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="N5" s="36" t="s">
+      <c r="N5" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="O5" s="36" t="s">
+      <c r="O5" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="P5" s="36" t="s">
+      <c r="P5" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="Q5" s="12" t="s">
+      <c r="Q5" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="R5" s="12" t="s">
+      <c r="R5" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="13.5">
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="M6" s="36" t="s">
+      <c r="M6" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="N6" s="15" t="s">
+      <c r="N6" s="11" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="13.5">
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="11" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="13.5">
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="M8" s="36" t="s">
+      <c r="M8" s="28" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:20" ht="25">
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M9" s="36" t="s">
+      <c r="M9" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="N9" s="15" t="s">
+      <c r="N9" s="11" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="13.5">
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="M10" s="36" t="s">
+      <c r="M10" s="28" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="13.5">
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H11" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="M11" s="36" t="s">
+      <c r="M11" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="N11" s="15" t="s">
+      <c r="N11" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="O11" s="36" t="s">
+      <c r="O11" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="P11" s="36" t="s">
+      <c r="P11" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="Q11" s="12" t="s">
+      <c r="Q11" s="8" t="s">
         <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" ht="25">
+      <c r="B12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="M12" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2678,7 +2726,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D40A82D-F7C3-47FE-9509-9F568C613B0F}">
-  <dimension ref="A1:D179"/>
+  <dimension ref="A1:D178"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="255.7265625" style="1" bestFit="1" customWidth="1"/>
@@ -2686,45 +2734,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="13.5">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="25" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="2"/>
     </row>
-    <row r="14" spans="1:1">
-      <c r="A14" s="4"/>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" s="4"/>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="4"/>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="4"/>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="4"/>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="4"/>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="5"/>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="4"/>
-    </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="6"/>
+      <c r="A22" s="3"/>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="6"/>
+      <c r="A23" s="3"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="6"/>
+      <c r="A24" s="3"/>
     </row>
     <row r="25" spans="1:4">
       <c r="D25">
@@ -2732,92 +2756,80 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="4"/>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="4"/>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="4"/>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="4"/>
-    </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="7"/>
+      <c r="A30" s="3"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="7"/>
+      <c r="A31" s="3"/>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="7"/>
+      <c r="A32" s="3"/>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="7"/>
+      <c r="A33" s="3"/>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="7"/>
+      <c r="A34" s="3"/>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="7"/>
+      <c r="A35" s="3"/>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="2"/>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="7"/>
+      <c r="A39" s="3"/>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" s="7"/>
+      <c r="A40" s="3"/>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" s="7"/>
+      <c r="A41" s="3"/>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="7"/>
+      <c r="A42" s="3"/>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" s="7"/>
+      <c r="A43" s="3"/>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" s="7"/>
+      <c r="A44" s="3"/>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" s="7"/>
+      <c r="A45" s="3"/>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" s="7"/>
+      <c r="A46" s="3"/>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" s="7"/>
+      <c r="A47" s="3"/>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="7"/>
+      <c r="A48" s="3"/>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="7"/>
+      <c r="A49" s="3"/>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="7"/>
+      <c r="A50" s="3"/>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="7"/>
+      <c r="A51" s="3"/>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" s="7"/>
+      <c r="A52" s="3"/>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" s="7"/>
+      <c r="A53" s="3"/>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="7"/>
+      <c r="A54" s="3"/>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" s="7"/>
+      <c r="A55" s="3"/>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" s="7"/>
+      <c r="A56" s="3"/>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="2"/>
@@ -2829,46 +2841,25 @@
       <c r="A61" s="2"/>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="7"/>
-    </row>
-    <row r="83" spans="1:1">
-      <c r="A83" s="4"/>
+      <c r="A74" s="3"/>
     </row>
     <row r="144" spans="1:1">
-      <c r="A144" s="7"/>
+      <c r="A144" s="3"/>
     </row>
     <row r="145" spans="1:1">
-      <c r="A145" s="7"/>
+      <c r="A145" s="3"/>
     </row>
     <row r="146" spans="1:1">
-      <c r="A146" s="7"/>
+      <c r="A146" s="3"/>
     </row>
     <row r="147" spans="1:1">
-      <c r="A147" s="7"/>
-    </row>
-    <row r="164" spans="1:1">
-      <c r="A164" s="4"/>
-    </row>
-    <row r="165" spans="1:1">
-      <c r="A165" s="3"/>
-    </row>
-    <row r="166" spans="1:1">
-      <c r="A166" s="3"/>
-    </row>
-    <row r="167" spans="1:1">
-      <c r="A167" s="3"/>
-    </row>
-    <row r="169" spans="1:1">
-      <c r="A169" s="3"/>
+      <c r="A147" s="3"/>
     </row>
     <row r="177" spans="1:1">
-      <c r="A177" s="7"/>
+      <c r="A177" s="3"/>
     </row>
     <row r="178" spans="1:1">
-      <c r="A178" s="7"/>
-    </row>
-    <row r="179" spans="1:1">
-      <c r="A179" s="4"/>
+      <c r="A178" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2884,160 +2875,160 @@
   <sheetFormatPr defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="11.453125" customWidth="1"/>
-    <col min="2" max="2" width="67.81640625" style="19" customWidth="1"/>
+    <col min="2" max="2" width="67.81640625" style="15" customWidth="1"/>
     <col min="3" max="3" width="24.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="13">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="13" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="13">
-      <c r="A2" s="18"/>
-      <c r="B2" s="19" t="s">
+      <c r="A2" s="14"/>
+      <c r="B2" s="15" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="13">
-      <c r="A3" s="20"/>
-      <c r="B3" s="19" t="s">
+      <c r="A3" s="16"/>
+      <c r="B3" s="15" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="13">
-      <c r="A4" s="21"/>
-      <c r="B4" s="19" t="s">
+      <c r="A4" s="17"/>
+      <c r="B4" s="15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="13">
-      <c r="A5" s="22"/>
-      <c r="B5" s="19" t="s">
+      <c r="A5" s="18"/>
+      <c r="B5" s="15" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="25.5" thickBot="1">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="19" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="12.75" customHeight="1">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="29" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="26.25" customHeight="1" thickBot="1">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="38"/>
+      <c r="C9" s="30"/>
     </row>
     <row r="10" spans="1:3" ht="25">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="15" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="13">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="13">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="24" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="13">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="24" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="25">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="13">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="19"/>
+      <c r="C15" s="15"/>
     </row>
     <row r="16" spans="1:3" ht="25">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="15" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="25">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="25">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="13">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="13" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="15" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="15" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="13">
-      <c r="B27" s="17"/>
+      <c r="B27" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat: add Kaplan-Meier survival plot vignette with gridify
- Refactor sample_titles2.xlsx: remove unused sheets, keep footer, footnote, description
- Add data dependencies: st_titles.xls and adam_adtte.xpt for vignette execution
- Create f_km.Rmd vignette demonstrating:
  * Survival analysis workflow with survminer
  * Figure annotation using gridify
  * Metadata integration with tflmetaR
- Generate example PDF outputs: f_surv_gridify.pdf and f_surv_tflmetar.pdf
</commit_message>
<xml_diff>
--- a/inst/extdata/sample_titles2.xlsx
+++ b/inst/extdata/sample_titles2.xlsx
@@ -1,34 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u066227\TFootr\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lancheng/Developer/UCB/tflmetaR/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77498BA8-4F73-4E04-BA1A-DCCCE046BBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A93EB843-F3EE-7449-A4C6-4EEC7A998999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{30221CC8-E0E7-4D3A-9A2D-9EE88E0E375F}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{30221CC8-E0E7-4D3A-9A2D-9EE88E0E375F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="footer" sheetId="6" r:id="rId2"/>
-    <sheet name="Footnotes" sheetId="2" r:id="rId3"/>
-    <sheet name="Descriptions" sheetId="4" r:id="rId4"/>
-    <sheet name="header" sheetId="5" r:id="rId5"/>
+    <sheet name="footer" sheetId="6" r:id="rId1"/>
+    <sheet name="Footnotes" sheetId="2" r:id="rId2"/>
+    <sheet name="Descriptions" sheetId="4" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">footer!$A$1:$T$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$2</definedName>
-    <definedName name="_Toc371317489" localSheetId="1">footer!#REF!</definedName>
-    <definedName name="_Toc371317489" localSheetId="0">Sheet1!#REF!</definedName>
-    <definedName name="_Toc424966764" localSheetId="1">footer!#REF!</definedName>
-    <definedName name="_Toc424966764" localSheetId="0">Sheet1!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">footer!$A$1:$T$2</definedName>
+    <definedName name="_Toc371317489" localSheetId="0">footer!#REF!</definedName>
+    <definedName name="_Toc424966764" localSheetId="0">footer!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="114">
   <si>
     <t>Pgmname</t>
   </si>
@@ -355,42 +350,6 @@
   </si>
   <si>
     <t>sample</t>
-  </si>
-  <si>
-    <t>UCB</t>
-  </si>
-  <si>
-    <t>MT-1621-ISE</t>
-  </si>
-  <si>
-    <t>CONFIDENTIAL</t>
-  </si>
-  <si>
-    <t>UL1</t>
-  </si>
-  <si>
-    <t>UL2</t>
-  </si>
-  <si>
-    <t>UL3</t>
-  </si>
-  <si>
-    <t>UR1</t>
-  </si>
-  <si>
-    <t>UR2</t>
-  </si>
-  <si>
-    <t>UR3</t>
-  </si>
-  <si>
-    <t>VERSION: FINAL</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>test2</t>
   </si>
   <si>
     <t>t_dm_m</t>
@@ -1896,31 +1855,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A371EE0A-5DB3-4461-B688-3161B666531D}">
-  <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57BBBF2B-056A-4DC3-A47F-4EB17BAEC258}">
+  <dimension ref="A1:T12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="26.6328125" style="8" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" style="9" customWidth="1"/>
-    <col min="4" max="5" width="14.7265625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="24.54296875" style="9" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="51.54296875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="27.453125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" style="8" customWidth="1"/>
-    <col min="12" max="12" width="9.1796875" style="8"/>
+    <col min="1" max="1" width="26.6640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" style="9" customWidth="1"/>
+    <col min="4" max="5" width="14.6640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="24.5" style="9" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="51.5" style="11" customWidth="1"/>
+    <col min="9" max="9" width="27.5" style="8" customWidth="1"/>
+    <col min="10" max="10" width="17.33203125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="12.1640625" style="8" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" style="8"/>
     <col min="13" max="13" width="40" style="11" customWidth="1"/>
-    <col min="14" max="14" width="39.26953125" style="11" customWidth="1"/>
-    <col min="15" max="15" width="37.1796875" style="11" customWidth="1"/>
-    <col min="16" max="16" width="30.54296875" style="8" customWidth="1"/>
-    <col min="17" max="17" width="27.1796875" style="8" customWidth="1"/>
-    <col min="18" max="18" width="126" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.1796875" style="8"/>
+    <col min="14" max="14" width="39.33203125" style="11" customWidth="1"/>
+    <col min="15" max="15" width="37.1640625" style="11" customWidth="1"/>
+    <col min="16" max="16" width="30.5" style="8" customWidth="1"/>
+    <col min="17" max="17" width="27.1640625" style="8" customWidth="1"/>
+    <col min="18" max="18" width="28.33203125" style="8" customWidth="1"/>
+    <col min="19" max="16384" width="9.1640625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="4" customFormat="1" ht="13">
+    <row r="1" spans="1:20" s="4" customFormat="1" ht="14">
       <c r="A1" s="4" t="s">
         <v>97</v>
       </c>
@@ -1982,7 +1941,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="27" customFormat="1" ht="25.5">
+    <row r="2" spans="1:20" s="27" customFormat="1" ht="28">
       <c r="A2" s="26" t="s">
         <v>48</v>
       </c>
@@ -2021,7 +1980,7 @@
       <c r="S2" s="7"/>
       <c r="T2" s="7"/>
     </row>
-    <row r="3" spans="1:20" ht="25">
+    <row r="3" spans="1:20" ht="28">
       <c r="B3" s="9" t="s">
         <v>79</v>
       </c>
@@ -2050,7 +2009,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="27">
+    <row r="4" spans="1:20" ht="30">
       <c r="C4" s="9" t="s">
         <v>54</v>
       </c>
@@ -2088,7 +2047,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="13.5">
+    <row r="5" spans="1:20" ht="15">
       <c r="C5" s="9" t="s">
         <v>59</v>
       </c>
@@ -2126,7 +2085,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="13.5">
+    <row r="6" spans="1:20" ht="15">
       <c r="C6" s="9" t="s">
         <v>85</v>
       </c>
@@ -2152,7 +2111,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="13.5">
+    <row r="7" spans="1:20" ht="15">
       <c r="C7" s="9" t="s">
         <v>69</v>
       </c>
@@ -2172,7 +2131,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="13.5">
+    <row r="8" spans="1:20" ht="15">
       <c r="C8" s="9" t="s">
         <v>72</v>
       </c>
@@ -2195,7 +2154,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="25">
+    <row r="9" spans="1:20" ht="28">
       <c r="C9" s="9" t="s">
         <v>74</v>
       </c>
@@ -2221,7 +2180,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="13.5">
+    <row r="10" spans="1:20" ht="15">
       <c r="C10" s="9" t="s">
         <v>76</v>
       </c>
@@ -2244,30 +2203,30 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="13.5">
+    <row r="11" spans="1:20" ht="15">
       <c r="B11" s="9" t="s">
         <v>79</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>51</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="M11" s="28" t="s">
         <v>95</v>
@@ -2285,435 +2244,36 @@
         <v>96</v>
       </c>
     </row>
-  </sheetData>
-  <autoFilter ref="A1:T2" xr:uid="{36D5F3F9-4062-4A10-8353-60238514C17B}"/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <headerFooter alignWithMargins="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57BBBF2B-056A-4DC3-A47F-4EB17BAEC258}">
-  <dimension ref="A1:T12"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5"/>
-  <cols>
-    <col min="1" max="1" width="26.6328125" style="8" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" style="9" customWidth="1"/>
-    <col min="4" max="5" width="14.7265625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="24.54296875" style="9" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="51.54296875" style="11" customWidth="1"/>
-    <col min="9" max="9" width="27.453125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
-    <col min="11" max="11" width="12.1796875" style="8" customWidth="1"/>
-    <col min="12" max="12" width="9.1796875" style="8"/>
-    <col min="13" max="13" width="40" style="11" customWidth="1"/>
-    <col min="14" max="14" width="39.26953125" style="11" customWidth="1"/>
-    <col min="15" max="15" width="37.1796875" style="11" customWidth="1"/>
-    <col min="16" max="16" width="30.54296875" style="8" customWidth="1"/>
-    <col min="17" max="17" width="27.1796875" style="8" customWidth="1"/>
-    <col min="18" max="18" width="28.26953125" style="8" customWidth="1"/>
-    <col min="19" max="16384" width="9.1796875" style="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:20" s="4" customFormat="1" ht="13">
-      <c r="A1" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" s="27" customFormat="1" ht="25.5">
-      <c r="A2" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="7"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="6" t="str">
-        <f>[1]Footnotes!A1</f>
-        <v>Footnotes</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
-      <c r="S2" s="7"/>
-      <c r="T2" s="7"/>
-    </row>
-    <row r="3" spans="1:20" ht="25">
-      <c r="B3" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="M3" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="N3" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" ht="27">
-      <c r="C4" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="M4" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="O4" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="P4" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q4" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="13.5">
-      <c r="C5" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="M5" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="N5" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="O5" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="P5" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q5" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="R5" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" ht="13.5">
-      <c r="C6" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="M6" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" ht="13.5">
-      <c r="C7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="13.5">
-      <c r="C8" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="M8" s="28" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" ht="25">
-      <c r="C9" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="M9" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" ht="13.5">
-      <c r="C10" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="M10" s="28" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" ht="13.5">
-      <c r="B11" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="9" t="s">
+    <row r="12" spans="1:20" ht="28">
+      <c r="B12" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" s="7" t="s">
+      <c r="M12" s="28" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="N12" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="O12" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="M11" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="N11" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="O11" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="P11" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q11" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" ht="25">
-      <c r="B12" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="M12" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="N12" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="O12" s="11" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2724,16 +2284,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D40A82D-F7C3-47FE-9509-9F568C613B0F}">
   <dimension ref="A1:D178"/>
-  <sheetFormatPr defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="255.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.1796875" customWidth="1"/>
+    <col min="1" max="1" width="255.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="13.5">
+    <row r="1" spans="1:1">
       <c r="A1" s="25" t="s">
         <v>47</v>
       </c>
@@ -2869,17 +2429,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7B55FF-88FF-47FD-9DBC-90367C69836D}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="11.453125" customWidth="1"/>
-    <col min="2" max="2" width="67.81640625" style="15" customWidth="1"/>
-    <col min="3" max="3" width="24.453125" customWidth="1"/>
+    <col min="1" max="1" width="11.5" customWidth="1"/>
+    <col min="2" max="2" width="67.83203125" style="15" customWidth="1"/>
+    <col min="3" max="3" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13">
+    <row r="1" spans="1:3" ht="14">
       <c r="A1" s="12" t="s">
         <v>22</v>
       </c>
@@ -2887,31 +2447,31 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="13">
+    <row r="2" spans="1:3" ht="14">
       <c r="A2" s="14"/>
       <c r="B2" s="15" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="13">
+    <row r="3" spans="1:3" ht="14">
       <c r="A3" s="16"/>
       <c r="B3" s="15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13">
+    <row r="4" spans="1:3" ht="14">
       <c r="A4" s="17"/>
       <c r="B4" s="15" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="13">
+    <row r="5" spans="1:3" ht="14">
       <c r="A5" s="18"/>
       <c r="B5" s="15" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="25.5" thickBot="1">
+    <row r="7" spans="1:3" ht="29" thickBot="1">
       <c r="A7" s="17" t="s">
         <v>28</v>
       </c>
@@ -2939,7 +2499,7 @@
       </c>
       <c r="C9" s="30"/>
     </row>
-    <row r="10" spans="1:3" ht="25">
+    <row r="10" spans="1:3" ht="28">
       <c r="A10" s="14" t="s">
         <v>1</v>
       </c>
@@ -2947,7 +2507,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13">
+    <row r="11" spans="1:3" ht="14">
       <c r="A11" s="14" t="s">
         <v>34</v>
       </c>
@@ -2955,7 +2515,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="13">
+    <row r="12" spans="1:3">
       <c r="A12" s="14" t="s">
         <v>36</v>
       </c>
@@ -2963,7 +2523,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13">
+    <row r="13" spans="1:3">
       <c r="A13" s="17" t="s">
         <v>10</v>
       </c>
@@ -2971,7 +2531,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="25">
+    <row r="14" spans="1:3" ht="28">
       <c r="A14" s="17" t="s">
         <v>11</v>
       </c>
@@ -2979,7 +2539,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13">
+    <row r="15" spans="1:3" ht="14">
       <c r="A15" s="17" t="s">
         <v>12</v>
       </c>
@@ -2988,7 +2548,7 @@
       </c>
       <c r="C15" s="15"/>
     </row>
-    <row r="16" spans="1:3" ht="25">
+    <row r="16" spans="1:3" ht="28">
       <c r="A16" s="17" t="s">
         <v>13</v>
       </c>
@@ -2996,7 +2556,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="25">
+    <row r="17" spans="1:2" ht="28">
       <c r="A17" s="18" t="s">
         <v>14</v>
       </c>
@@ -3004,7 +2564,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="25">
+    <row r="18" spans="1:2" ht="28">
       <c r="A18" s="18" t="s">
         <v>15</v>
       </c>
@@ -3012,22 +2572,22 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="13">
+    <row r="22" spans="1:2" ht="14">
       <c r="B22" s="13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" ht="14">
       <c r="B23" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" ht="14">
       <c r="B24" s="15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="13">
+    <row r="27" spans="1:2">
       <c r="B27" s="13"/>
     </row>
   </sheetData>
@@ -3038,543 +2598,4 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4CA7B3B-3FD8-4486-ACD0-C11FB97FCEF0}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
-  <cols>
-    <col min="3" max="3" width="11.08984375" customWidth="1"/>
-    <col min="6" max="6" width="11.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="I6" location="RELREC!A1" display="RELREC" xr:uid="{3503CC0B-9198-4F60-810B-FC408BF4C3A3}"/>
-    <hyperlink ref="I7" location="MB!A1" display="MB" xr:uid="{F008118A-4485-4E6F-992B-9CB6B8A8AA63}"/>
-    <hyperlink ref="I14" location="RE!A1" display="RE" xr:uid="{AA1DF241-67D9-4FF1-A590-0C60515FA079}"/>
-    <hyperlink ref="I1" location="SUPP!A1" display="SUPP" xr:uid="{906AEEAD-CA15-4274-BD23-9DB659EB4DD4}"/>
-    <hyperlink ref="I11" location="PE!A1" display="PE" xr:uid="{A156BDC6-B0BB-4724-A0C2-18A03D409EE2}"/>
-    <hyperlink ref="I8" location="SUPP!A1" display="SUPP" xr:uid="{64EF6DBF-7BDB-4C0C-88AB-CF9936DC9DE8}"/>
-    <hyperlink ref="I9" location="SC!A1" display="SC" xr:uid="{D55A46AC-CEC2-4697-A516-FB9682CEC916}"/>
-    <hyperlink ref="I32" location="SC!A1" display="SC!A1" xr:uid="{94F93248-A02E-4DFF-83D9-AD31656B88CA}"/>
-    <hyperlink ref="I2" location="RE!A1" display="RE" xr:uid="{3FFCAED1-E810-4DF3-AA1E-EB087DF9A80A}"/>
-    <hyperlink ref="I4" location="FA!A1" display="FA" xr:uid="{31532BF4-A686-450B-B350-8C8AC83BD7AC}"/>
-    <hyperlink ref="I5" location="FA!A1" display="FA" xr:uid="{7677A654-D951-49CE-A1E2-7B3E730C30C2}"/>
-    <hyperlink ref="I10" location="MS!A1" display="MS" xr:uid="{6788F4EA-51E7-4FC8-A63D-B745ED811D18}"/>
-    <hyperlink ref="I3" location="VS!A1" display="VS" xr:uid="{9625FF7C-B5C4-4FD7-AC20-3805410ED74C}"/>
-    <hyperlink ref="I33" location="SC!A1" display="SC!A1" xr:uid="{1C9749B5-C99C-4041-99B1-D9F23D00F253}"/>
-    <hyperlink ref="I12:I13" location="PE!A1" display="PE" xr:uid="{5F2AB33E-DE29-44A5-A753-32974DABE98F}"/>
-    <hyperlink ref="I16:I21" location="SC!A1" display="SC" xr:uid="{AD7D2370-6175-4809-8EFF-DFDD0ECEE8F2}"/>
-    <hyperlink ref="I25" location="SC!A1" display="SC!A1" xr:uid="{654EDCDC-CBA0-448E-8D66-4368A20F9840}"/>
-    <hyperlink ref="I23" location="SC!A1" display="SC!A1" xr:uid="{475DD5A5-3D50-41BF-A123-57BADF842106}"/>
-    <hyperlink ref="I24" location="SC!A1" display="SC!A1" xr:uid="{4EDA0462-2B7F-494E-8F86-9025949B817D}"/>
-    <hyperlink ref="I22" location="SC!A1" display="SC!A1" xr:uid="{946B137C-89F1-4417-B2B2-D2EBD216F11E}"/>
-    <hyperlink ref="I19" location="SC!A1" display="SC!A1" xr:uid="{494445E9-BB61-4E12-9C0E-F0D5AA6348D9}"/>
-    <hyperlink ref="I15" location="SC!A1" display="SC!A1" xr:uid="{A547C4F9-1842-49B6-9E45-4A4A87C396D5}"/>
-    <hyperlink ref="I16" location="SC!A1" display="SC!A1" xr:uid="{9309FFB3-A08F-4522-956F-C1689A0A951D}"/>
-    <hyperlink ref="I17" location="SC!A1" display="SC!A1" xr:uid="{E2F10D94-BF59-43F3-B091-9779EC76A9C8}"/>
-    <hyperlink ref="I18" location="SC!A1" display="SC!A1" xr:uid="{35EA46ED-9D1D-42EC-B2A8-962A318A36EB}"/>
-    <hyperlink ref="I20" location="SC!A1" display="SC!A1" xr:uid="{38E0DA44-23F0-457D-9A7A-03EAF14193BB}"/>
-    <hyperlink ref="I28" location="SC!A1" display="SC!A1" xr:uid="{F11677F8-A485-4BE8-ABAC-067C3DC130A9}"/>
-    <hyperlink ref="I29" location="SC!A1" display="SC!A1" xr:uid="{01F7E7EA-AD8C-43EA-BF9E-0FFBE39A66EB}"/>
-    <hyperlink ref="N15" location="SC!A1" display="SC" xr:uid="{18D3360B-62D4-40A2-85C4-6C5EC706F07E}"/>
-    <hyperlink ref="N32" location="SC!A1" display="SC" xr:uid="{7F1427F5-3F87-4DD3-BBEF-6FE1C98191F9}"/>
-    <hyperlink ref="N16:N21" location="SC!A1" display="SC" xr:uid="{965EAA68-A4A3-44D2-80C7-CAA68A5867CA}"/>
-    <hyperlink ref="N19" location="SC!A1" display="SC" xr:uid="{89885848-EF31-49EE-935D-6EF034E7FA3B}"/>
-    <hyperlink ref="N22" location="SC!A1" display="SC" xr:uid="{E03EBAC3-4850-47CD-8FE9-D9CED72244D8}"/>
-    <hyperlink ref="N25" location="SC!A1" display="SC" xr:uid="{4D4FB9CC-F9BD-4435-BDFB-85C2D1E8CA24}"/>
-    <hyperlink ref="N23" location="AE!A1" display="AE" xr:uid="{67BB241D-F09A-432E-A59C-0718EEF2518E}"/>
-    <hyperlink ref="N24" location="SC!A1" display="SC" xr:uid="{226CFD4E-1646-4079-B2CA-27CC1055B6BA}"/>
-    <hyperlink ref="I21" location="SC!A1" display="SC!A1" xr:uid="{BAC21FA6-343E-4C01-BE1B-5D3872EA5638}"/>
-    <hyperlink ref="I30" location="SC!A1" display="SC!A1" xr:uid="{C1EE70A3-727C-4020-949F-7B4EA1A6D5DB}"/>
-    <hyperlink ref="I31" location="SC!A1" display="SC!A1" xr:uid="{853FEE67-9C78-42D7-B9A8-B61A2DFF41A5}"/>
-    <hyperlink ref="N17" location="SC!A1" display="SC" xr:uid="{2B5D285A-858A-4FB3-91CA-51936F2576D8}"/>
-    <hyperlink ref="N18:N23" location="SC!A1" display="SC" xr:uid="{2F9F772A-28A5-4723-8F1D-00D0A0B3EC42}"/>
-    <hyperlink ref="N21" location="SC!A1" display="SC" xr:uid="{D17C82E1-733E-451F-9BBB-0F5BDA9B0A1C}"/>
-    <hyperlink ref="N27" location="SC!A1" display="SC" xr:uid="{AD18DE75-C71D-4940-B7D6-2AA3B7CE3EF9}"/>
-    <hyperlink ref="N26" location="AE!A1" display="AE" xr:uid="{1754421A-87AA-44F8-A06E-6C8B801E1F5E}"/>
-    <hyperlink ref="N18" location="SC!A1" display="SC" xr:uid="{7D01B36D-2B98-47B1-9243-562ABF86996E}"/>
-    <hyperlink ref="N19:N24" location="SC!A1" display="SC" xr:uid="{9D93FA5A-1494-48DC-9221-1565B25F2C07}"/>
-    <hyperlink ref="N28" location="SC!A1" display="SC" xr:uid="{C38F99A5-8DA0-4FEC-B878-47F0A39484D1}"/>
-    <hyperlink ref="I27" location="SC!A1" display="SC!A1" xr:uid="{5C5E0AB1-4E2F-4C3E-BD7A-12B8E6D31527}"/>
-    <hyperlink ref="N20" location="SC!A1" display="SC" xr:uid="{E44C4186-A9FB-4991-A13F-630299D02002}"/>
-    <hyperlink ref="N21:N26" location="SC!A1" display="SC" xr:uid="{A1804633-D8E1-4D73-8BD1-0DA0B027DCC2}"/>
-    <hyperlink ref="N30" location="SC!A1" display="SC" xr:uid="{35EF6E1A-9C71-4F0F-AC2F-D6DD3906DD69}"/>
-    <hyperlink ref="N29" location="SC!A1" display="SC" xr:uid="{A72D0018-0129-499C-9DB0-637FD15682E7}"/>
-    <hyperlink ref="I26" location="SC!A1" display="SC!A1" xr:uid="{006D91E4-C36E-446F-8763-E0DD450AFC2D}"/>
-    <hyperlink ref="I34" location="SC!A1" display="SC!A1" xr:uid="{8D2A8E93-FE90-4FCA-98FF-4C868DDDA12D}"/>
-    <hyperlink ref="N22:N27" location="SC!A1" display="SC" xr:uid="{FAD8B0D7-EE08-4962-855D-762D2E1CBA6E}"/>
-    <hyperlink ref="N31" location="SC!A1" display="SC" xr:uid="{9D361774-D007-4F53-9467-4208C89A3A91}"/>
-    <hyperlink ref="I36" location="SC!A1" display="SC!A1" xr:uid="{6C5025C6-DB9D-4953-BF4D-BAE341F13B07}"/>
-    <hyperlink ref="I37" location="SC!A1" display="SC!A1" xr:uid="{9106CDF8-E147-4FA7-8DFC-58A7F1A24529}"/>
-    <hyperlink ref="N25:N30" location="SC!A1" display="SC" xr:uid="{15E319C2-1041-40B4-8801-4D5E89AAFB6D}"/>
-    <hyperlink ref="I39" location="SC!A1" display="SC!A1" xr:uid="{210CCF81-9556-4BFC-8B83-5ACF3F6009E9}"/>
-    <hyperlink ref="I40" location="SC!A1" display="SC!A1" xr:uid="{EC0E36F5-C2BF-456C-B7D1-7225419DF872}"/>
-    <hyperlink ref="N28:N32" location="SC!A1" display="SC" xr:uid="{41E29174-FD8B-4190-ABF7-C1D9BE423ED0}"/>
-    <hyperlink ref="I35" location="SC!A1" display="SC!A1" xr:uid="{8FF4F7A6-6169-4E0B-9D0E-2912A10FC902}"/>
-    <hyperlink ref="I41" location="SC!A1" display="SC!A1" xr:uid="{2051BE24-8DD8-4D81-9B67-8C7274CFA06D}"/>
-    <hyperlink ref="N30:N34" location="SC!A1" display="SC" xr:uid="{3B133F73-B00B-4632-9309-153BC2312814}"/>
-    <hyperlink ref="I42" location="SC!A1" display="SC!A1" xr:uid="{98804136-7DD4-4489-B479-5EBB123D7386}"/>
-    <hyperlink ref="N31:N35" location="SC!A1" display="SC" xr:uid="{44224ECF-DBE8-4089-A13B-4B96D81F7B3B}"/>
-    <hyperlink ref="I38" location="SC!A1" display="SC!A1" xr:uid="{688C6AC0-B8B9-4BD0-9163-ADC3753DBDDC}"/>
-    <hyperlink ref="I43" location="SC!A1" display="SC!A1" xr:uid="{889B457A-8447-437C-B02B-5BF02EF5D897}"/>
-    <hyperlink ref="I44" location="SC!A1" display="SC!A1" xr:uid="{027E7C4E-FC22-4A06-8A1E-6905360D2DE7}"/>
-    <hyperlink ref="I45" location="SC!A1" display="SC!A1" xr:uid="{146F418F-C53E-42AC-AE37-1AC2ED2145F8}"/>
-    <hyperlink ref="I46" location="SC!A1" display="SC!A1" xr:uid="{B5E30194-47EE-49BF-95C6-3B38C12B06E9}"/>
-    <hyperlink ref="I47" location="SC!A1" display="SC!A1" xr:uid="{C816ABA8-5C37-43E8-B973-6961467348C3}"/>
-    <hyperlink ref="I48" location="SC!A1" display="SC!A1" xr:uid="{75DB9A2D-3D5A-4256-9CC2-C64E316CAB32}"/>
-    <hyperlink ref="I49" location="SC!A1" display="SC!A1" xr:uid="{8968758A-8CCA-469B-8383-89F83928EA36}"/>
-    <hyperlink ref="I50" location="SC!A1" display="SC!A1" xr:uid="{0E3C3AB3-3124-497A-9BB8-464165A86ECC}"/>
-    <hyperlink ref="I51" location="SC!A1" display="SC!A1" xr:uid="{27381B41-DA1F-4C61-B17E-1F0B7513E456}"/>
-    <hyperlink ref="I52" location="SC!A1" display="SC!A1" xr:uid="{301ACEE0-A2E5-497B-B9FD-2805E9F93102}"/>
-    <hyperlink ref="I53" location="SC!A1" display="SC!A1" xr:uid="{10E68F16-75EA-4CEF-A6EA-73143433B351}"/>
-    <hyperlink ref="I54" location="SC!A1" display="SC!A1" xr:uid="{24E8EEAE-2956-4169-9B84-A18DC5F803F2}"/>
-    <hyperlink ref="N59" location="SC!A1" display="SC" xr:uid="{6614BBD4-2CC8-44ED-AF16-A8840E320DB4}"/>
-    <hyperlink ref="I55" location="SC!A1" display="SC!A1" xr:uid="{3B20FC1E-0595-4610-A9A5-240B76843FE0}"/>
-    <hyperlink ref="I56" location="SC!A1" display="SC!A1" xr:uid="{A5E4DE90-11FD-4390-8FDE-D186A5087BF2}"/>
-    <hyperlink ref="N60" location="AE!A1" display="AE" xr:uid="{63F06786-CCA0-4D09-BFBC-60A25C00880F}"/>
-    <hyperlink ref="N61" location="SC!A1" display="SC" xr:uid="{46BC878C-48DA-47B9-ADA3-D3E2C64ACC0D}"/>
-    <hyperlink ref="I57" location="SC!A1" display="SC!A1" xr:uid="{790D2770-9459-4519-A876-BE31D030D9D5}"/>
-    <hyperlink ref="N62" location="AE!A1" display="AE" xr:uid="{EC9746C3-D861-4690-BAB3-74231B490CB0}"/>
-    <hyperlink ref="I58" location="SC!A1" display="SC!A1" xr:uid="{9F01BC4E-6D08-4648-837A-5EB13290C39E}"/>
-    <hyperlink ref="I59" location="AE!A1" display="AE!A1" xr:uid="{76A39B50-8086-4FFC-BE83-F5D1F03AAFCB}"/>
-    <hyperlink ref="N63" location="AE!A1" display="AE" xr:uid="{9F492687-D495-462D-B6B4-46480CB171AE}"/>
-    <hyperlink ref="N64" location="CE!A1" display="CE" xr:uid="{496C9A5A-4748-44E0-AD25-50F220FC2A37}"/>
-    <hyperlink ref="I60" location="RE!A1" display="RE!A1" xr:uid="{BBE4F923-4120-4E68-B3FD-54793ACACEF1}"/>
-    <hyperlink ref="N65" location="RE!A1" display="RE" xr:uid="{295A95AE-8BDC-4D81-9C27-81ED98E42F98}"/>
-    <hyperlink ref="I61" location="CE!A1" display="CE!A1" xr:uid="{DAFAD91F-738F-4A0C-B4F2-8F3780E9BE66}"/>
-    <hyperlink ref="I62" location="RE!A1" display="RE!A1" xr:uid="{80A09244-6CA7-45C2-88E2-FCECBDF07F9C}"/>
-    <hyperlink ref="N66" location="RE!A1" display="RE" xr:uid="{CB33B786-D3ED-40BB-A6DC-3127008C0520}"/>
-    <hyperlink ref="N67" location="SC!A1" display="SC" xr:uid="{20D2DFA1-0285-4CA1-AB7D-2C6BF90575E7}"/>
-    <hyperlink ref="I63" location="RE!A1" display="RE!A1" xr:uid="{20091604-B99C-4D75-B2EE-47BDE03F7474}"/>
-    <hyperlink ref="N68" location="RE!A1" display="RE" xr:uid="{0C1C57B4-29CC-46B0-A050-50B1E7171B8E}"/>
-    <hyperlink ref="I64" location="RE!A1" display="RE!A1" xr:uid="{8F6563F6-46C5-47FA-A74F-9F31718D9151}"/>
-    <hyperlink ref="I65" location="RE!A1" display="RE!A1" xr:uid="{33D247EE-9947-4E9F-856C-D8727A5341E0}"/>
-    <hyperlink ref="N69" location="RE!A1" display="RE" xr:uid="{6D423903-2260-4D3F-876C-7255CC85A5E6}"/>
-    <hyperlink ref="N70" location="RE!A1" display="RE" xr:uid="{28A9FDC8-D8C5-450B-B96D-DA55303BAD84}"/>
-    <hyperlink ref="I66" location="RE!A1" display="RE!A1" xr:uid="{EF1E7FE4-43CD-4315-9163-EF47C44E0E67}"/>
-    <hyperlink ref="N71" location="SC!A1" display="SC" xr:uid="{08DCE6E5-12D6-49AD-AC55-64FE34A35CC5}"/>
-    <hyperlink ref="I67" location="SC!A1" display="SC!A1" xr:uid="{0D158FC7-3111-4441-9770-1494E0602D9C}"/>
-    <hyperlink ref="I68" location="SC!A1" display="SC!A1" xr:uid="{47D99793-53A6-49CF-A0B8-E1809FCDED7D}"/>
-    <hyperlink ref="N72" location="RE!A1" display="RE" xr:uid="{F05C2A14-26E8-4913-BC53-CA6934B68627}"/>
-    <hyperlink ref="N73" location="RE!A1" display="RE" xr:uid="{51B221CD-0362-4049-9D7B-3927219028A1}"/>
-    <hyperlink ref="N55:N60" location="SC!A1" display="SC" xr:uid="{3AB8FDEF-503E-47E4-9F18-58DEBF9CFC4E}"/>
-    <hyperlink ref="I69" location="SC!A1" display="SC!A1" xr:uid="{0BFA2BA0-A5E7-44ED-8454-EFF164AFAF4D}"/>
-    <hyperlink ref="I70" location="SC!A1" display="SC!A1" xr:uid="{39265F97-324F-4943-B073-56B910F89888}"/>
-    <hyperlink ref="I71" location="SC!A1" display="SC!A1" xr:uid="{EC1D21FA-E07E-42CF-A6AB-DE9B3452836F}"/>
-    <hyperlink ref="I72" location="AE!A1" display="AE!A1" xr:uid="{5F38BD4D-30D3-4085-B635-3D49ACE8E48F}"/>
-    <hyperlink ref="I74" location="CE!A1" display="CE!A1" xr:uid="{10507A21-2B96-43BB-B982-2E657BCABF52}"/>
-    <hyperlink ref="I80" location="RE!A1" display="RE!A1" xr:uid="{D713A62C-6D63-419F-A8F5-19D247C59018}"/>
-    <hyperlink ref="I81" location="RE!A1" display="RE!A1" xr:uid="{161E4E23-AF1C-4EB1-B55C-DEB600DDB942}"/>
-    <hyperlink ref="N84" location="RE!A1" display="RE" xr:uid="{8EC99D1B-69D6-4000-B54F-CFC81894625E}"/>
-    <hyperlink ref="N85" location="RE!A1" display="RE" xr:uid="{94EB3B41-D1AC-4C05-A391-92E8D58704CB}"/>
-    <hyperlink ref="N86" location="RE!A1" display="RE" xr:uid="{1174703C-DD45-4F16-943D-E909C4A63E99}"/>
-    <hyperlink ref="N68:N73" location="SC!A1" display="SC" xr:uid="{EDA7D651-A369-4712-8C3E-FB8969F259C4}"/>
-    <hyperlink ref="N74" location="SC!A1" display="SC" xr:uid="{9E69A374-54D3-4AAD-A945-360B5C483107}"/>
-    <hyperlink ref="N77" location="CE!A1" display="CE" xr:uid="{D683952D-91B5-49C7-9B64-9F3666EACF5F}"/>
-    <hyperlink ref="N75" location="AE!A1" display="AE" xr:uid="{DAA6B1B8-E902-41DD-B08E-13D34E5D25C1}"/>
-    <hyperlink ref="N76" location="AE!A1" display="AE" xr:uid="{765252CF-0D40-4D27-A9CB-A5DE5BAD71CD}"/>
-    <hyperlink ref="I88" location="SC!A1" display="SC!A1" xr:uid="{200697B6-7A16-4298-B40D-3D07932C8861}"/>
-    <hyperlink ref="I89" location="SC!A1" display="SC!A1" xr:uid="{623EFF12-259B-444F-8169-1048100485A8}"/>
-    <hyperlink ref="I90" location="SC!A1" display="SC!A1" xr:uid="{A73DAB2F-CAD7-4A0C-B668-CF90E089C572}"/>
-    <hyperlink ref="I91" location="SC!A1" display="SC!A1" xr:uid="{1AC10A13-8A24-4B11-B6E4-1F2DE8D99FF8}"/>
-    <hyperlink ref="I92" location="SC!A1" display="SC!A1" xr:uid="{99011AC3-4792-41F4-860E-F04C1E8F9257}"/>
-    <hyperlink ref="I93" location="AE!A1" display="AE!A1" xr:uid="{A2F2ADD6-85C7-4584-8499-A2C80A412019}"/>
-    <hyperlink ref="I95" location="SC!A1" display="SC!A1" xr:uid="{47BD150B-163B-4935-B9CD-AE206ACD7AE6}"/>
-    <hyperlink ref="I101" location="RE!A1" display="RE!A1" xr:uid="{44771E48-7EA2-4807-BEB5-2A4ADCCD1144}"/>
-    <hyperlink ref="I102" location="CE!A1" display="CE!A1" xr:uid="{A04096B4-F5CC-4646-8365-9A528E87B112}"/>
-    <hyperlink ref="N88" location="SC!A1" display="SC" xr:uid="{7B7D3770-C161-4A28-AB51-821004868F9C}"/>
-    <hyperlink ref="N105" location="CE!A1" display="CE" xr:uid="{019CEF93-26B7-4289-AA3F-E0CB63CB7620}"/>
-    <hyperlink ref="N106" location="RE!A1" display="RE" xr:uid="{8CDCA326-3B98-4A9E-B963-EC73FF43A6F3}"/>
-    <hyperlink ref="N107" location="RE!A1" display="RE" xr:uid="{006A3130-F3DC-4BD6-8DB1-F19F7AC10834}"/>
-    <hyperlink ref="N89:N94" location="SC!A1" display="SC" xr:uid="{06C20BD0-786D-48F7-ADB0-FF38C72F4603}"/>
-    <hyperlink ref="N92" location="SC!A1" display="SC" xr:uid="{A399CC6A-DC8A-4451-8495-BFB81096BA5D}"/>
-    <hyperlink ref="N95" location="SC!A1" display="SC" xr:uid="{62DC0D44-322A-4116-B86E-BFDE02CED157}"/>
-    <hyperlink ref="N98" location="CE!A1" display="CE" xr:uid="{04391598-99E3-42FC-9AC4-F8FDF9A2FFE3}"/>
-    <hyperlink ref="N96" location="AE!A1" display="AE" xr:uid="{92D42861-3D2D-4AD3-906F-D6BB0D6BE975}"/>
-    <hyperlink ref="N97" location="AE!A1" display="AE" xr:uid="{B2ACB69C-766B-43CB-B7B4-1D6DD85572A6}"/>
-    <hyperlink ref="I96" location="SC!A1" display="SC!A1" xr:uid="{9F7E6BB1-5C3D-48B1-807F-D81FFD9AB219}"/>
-    <hyperlink ref="I97" location="SC!A1" display="SC!A1" xr:uid="{3A35B468-C312-4A44-BB72-2EBF541F2171}"/>
-    <hyperlink ref="I98" location="SC!A1" display="SC!A1" xr:uid="{241C2954-624C-4A06-B600-5A47CB4DDA1E}"/>
-    <hyperlink ref="I99" location="SC!A1" display="SC!A1" xr:uid="{B28C082E-78CD-4CA8-8DA5-03540ECC5146}"/>
-    <hyperlink ref="I100" location="AE!A1" display="AE!A1" xr:uid="{F034EF11-2C37-414F-B05C-4EEB086F17E3}"/>
-    <hyperlink ref="I108" location="RE!A1" display="RE!A1" xr:uid="{4159808C-2996-4A7E-BDBB-0CB7932661A3}"/>
-    <hyperlink ref="I109" location="RE!A1" display="RE!A1" xr:uid="{3F1345DC-B1E0-43A2-8695-FF39AF90764A}"/>
-    <hyperlink ref="N112" location="RE!A1" display="RE" xr:uid="{AFC395BB-27A5-4917-88B4-1409A5C69EF8}"/>
-    <hyperlink ref="N113" location="RE!A1" display="RE" xr:uid="{71F2DFEF-62B2-4A29-ADA8-9B56D67CF766}"/>
-    <hyperlink ref="N114" location="RE!A1" display="RE" xr:uid="{D44EF772-5D76-42BB-A2B6-8B07219227E1}"/>
-    <hyperlink ref="N96:N101" location="SC!A1" display="SC" xr:uid="{53B1E094-34AE-40E7-88B0-A59887C3E669}"/>
-    <hyperlink ref="N99" location="SC!A1" display="SC" xr:uid="{A13924E8-5C6E-4BCB-97EF-667D2AF37B02}"/>
-    <hyperlink ref="N102" location="SC!A1" display="SC" xr:uid="{07A411F7-A7FD-463B-8EC7-2FC65F39F50D}"/>
-    <hyperlink ref="N103" location="AE!A1" display="AE" xr:uid="{D98B81F8-D915-4364-BCE2-A01164B12D72}"/>
-    <hyperlink ref="N104" location="AE!A1" display="AE" xr:uid="{535057C4-E636-44D6-8035-E7B8E96ABAE8}"/>
-    <hyperlink ref="I120" location="SC!A1" display="SC!A1" xr:uid="{7FC9E6B8-BEDB-4D13-987A-064B1AEBF8DB}"/>
-    <hyperlink ref="I121" location="SC!A1" display="SC!A1" xr:uid="{16CC204B-5319-427B-8867-17CAAB3E1B98}"/>
-    <hyperlink ref="I122" location="SC!A1" display="SC!A1" xr:uid="{26D628E7-D54D-479F-B902-8D652F5F982F}"/>
-    <hyperlink ref="I123" location="SC!A1" display="SC!A1" xr:uid="{E40B7535-5AB8-43BD-A3DC-55A96D882DE4}"/>
-    <hyperlink ref="I124" location="SC!A1" display="SC!A1" xr:uid="{E4581357-45F6-41BB-8963-A3B005BB88AB}"/>
-    <hyperlink ref="I125" location="SC!A1" display="SC!A1" xr:uid="{7297139B-FBCF-4189-8674-A5AA4657EDE2}"/>
-    <hyperlink ref="I127" location="SC!A1" display="SC!A1" xr:uid="{2A654727-FAF4-4EE2-AA90-5F19C38161DC}"/>
-    <hyperlink ref="I133" location="SC!A1" display="SC!A1" xr:uid="{3D47D105-76A3-4939-BC60-697BDBCFEA14}"/>
-    <hyperlink ref="I134" location="SC!A1" display="SC!A1" xr:uid="{2B2504DC-7110-4711-B072-3488F9CCEA45}"/>
-    <hyperlink ref="N120" location="SC!A1" display="SC" xr:uid="{7E1F14DD-6BA4-4BA3-8D6E-1721BC5BF3B7}"/>
-    <hyperlink ref="N137" location="SC!A1" display="SC" xr:uid="{CAF8D439-0C64-46D9-8F98-E8DD4FDD6584}"/>
-    <hyperlink ref="N138" location="SC!A1" display="SC" xr:uid="{88C4ABF8-7C77-4C90-8162-7B0EC2A2C9D7}"/>
-    <hyperlink ref="N139" location="AE!A1" display="AE" xr:uid="{AEF2A0FB-DDA2-46AE-8BFF-2F48E989CC9D}"/>
-    <hyperlink ref="N121:N126" location="SC!A1" display="SC" xr:uid="{C7EB1E5E-72E9-4866-AC18-A228B246A94D}"/>
-    <hyperlink ref="N124" location="SC!A1" display="SC" xr:uid="{405F416A-3CAB-42A1-B882-C874ED82B95F}"/>
-    <hyperlink ref="N127" location="SC!A1" display="SC" xr:uid="{F13374E6-DBB5-49EE-9AC4-3926BA33DD4E}"/>
-    <hyperlink ref="N130" location="SC!A1" display="SC" xr:uid="{27441C0E-C23B-449D-AB9B-3504427700B7}"/>
-    <hyperlink ref="N128" location="AE!A1" display="AE" xr:uid="{CFAE6B18-1C03-4BC5-9FCA-741B374E6C51}"/>
-    <hyperlink ref="N129" location="AE!A1" display="AE" xr:uid="{B59D9A76-324C-412E-AD8B-D55D06E38B08}"/>
-    <hyperlink ref="I126" location="SC!A1" display="SC!A1" xr:uid="{A2149FB3-578C-4833-AEE2-9A82FF2F3722}"/>
-    <hyperlink ref="I128" location="SC!A1" display="SC!A1" xr:uid="{05607723-FC2F-4013-916C-A235455D102F}"/>
-    <hyperlink ref="I130" location="SC!A1" display="SC!A1" xr:uid="{6B64ABFA-EB75-4830-958F-F27E7676403A}"/>
-    <hyperlink ref="I136" location="SC!A1" display="SC!A1" xr:uid="{C9ED0FE7-39E0-4D9C-B72C-B887228CC417}"/>
-    <hyperlink ref="I137" location="SC!A1" display="SC!A1" xr:uid="{55E502FC-A264-4CA6-BD0A-03E3B0F2BA92}"/>
-    <hyperlink ref="N123" location="SC!A1" display="SC" xr:uid="{D9519AD5-8162-4491-9E8C-903082972D73}"/>
-    <hyperlink ref="N140" location="SC!A1" display="SC" xr:uid="{C6763349-C241-44C1-8289-2E41DED9A419}"/>
-    <hyperlink ref="N141" location="AE!A1" display="AE" xr:uid="{A9EA7E0D-A835-4785-A23A-DA246C91AC6A}"/>
-    <hyperlink ref="N142" location="AE!A1" display="AE" xr:uid="{28E15711-DF67-426B-9108-1FB4AFFE2279}"/>
-    <hyperlink ref="N124:N129" location="SC!A1" display="SC" xr:uid="{5CEA0D2F-A30A-4659-A887-9B6ECD51437C}"/>
-    <hyperlink ref="N133" location="SC!A1" display="SC" xr:uid="{2B3C42F7-ABF8-41D1-A226-A68E78335435}"/>
-    <hyperlink ref="N131" location="SC!A1" display="SC" xr:uid="{F67ED0F5-1BD3-42C7-96D7-E50DEFB0B6AA}"/>
-    <hyperlink ref="N132" location="AE!A1" display="AE" xr:uid="{6D963A4C-23E5-44BE-9AE4-C7A831F1F12A}"/>
-    <hyperlink ref="I129" location="SC!A1" display="SC!A1" xr:uid="{67AEB233-D020-4546-9531-FBF0B27FC2A0}"/>
-    <hyperlink ref="I131" location="SC!A1" display="SC!A1" xr:uid="{B8D3B0A9-4FF7-4678-9451-9ABF7807C68C}"/>
-    <hyperlink ref="I132" location="SC!A1" display="SC!A1" xr:uid="{DE7F08C8-F54F-410B-9655-A99C5C790D89}"/>
-    <hyperlink ref="I140" location="CE!A1" display="CE!A1" xr:uid="{18BB66F0-C45D-4E1D-9827-A36354D19A49}"/>
-    <hyperlink ref="I141" location="RE!A1" display="RE!A1" xr:uid="{DBB07655-9878-4BBD-8832-B1A26714A60D}"/>
-    <hyperlink ref="N144" location="SC!A1" display="SC" xr:uid="{4CD43B6C-910D-4B1B-AC64-7B2D7314CFC6}"/>
-    <hyperlink ref="N145" location="RE!A1" display="RE" xr:uid="{55ABB867-A203-4128-850A-3F30162D7BC6}"/>
-    <hyperlink ref="N146" location="RE!A1" display="RE" xr:uid="{5B6FBE95-F121-43B2-8A46-D75DFFA93F72}"/>
-    <hyperlink ref="N128:N133" location="SC!A1" display="SC" xr:uid="{15C29BC3-3CAB-4631-BCA6-AE8DD3F1093A}"/>
-    <hyperlink ref="N134" location="SC!A1" display="SC" xr:uid="{C7500B1E-E766-431A-BF83-26DC0F449033}"/>
-    <hyperlink ref="N135" location="SC!A1" display="SC" xr:uid="{0BF8A126-4DE1-4592-B464-BA01DDF576B1}"/>
-    <hyperlink ref="N136" location="AE!A1" display="AE" xr:uid="{145DAC6C-79DD-4FC2-862F-C5A6C1F0E1EC}"/>
-    <hyperlink ref="I135" location="SC!A1" display="SC!A1" xr:uid="{3D4A110C-3807-4979-94F5-CDCA4C0E5E52}"/>
-    <hyperlink ref="I138" location="AE!A1" display="AE!A1" xr:uid="{7A9EEAD4-A3BA-41FE-BA1A-250B7D4B7BB6}"/>
-    <hyperlink ref="I144" location="SC!A1" display="SC!A1" xr:uid="{A6D03BDC-3A31-46F5-AD54-28F9625598A0}"/>
-    <hyperlink ref="I145" location="SC!A1" display="SC!A1" xr:uid="{F213B1AC-8186-44F2-B043-2B2F4938A25E}"/>
-    <hyperlink ref="N148" location="SC!A1" display="SC" xr:uid="{E5CF1703-80FD-4355-B9BC-4F65EFD9346F}"/>
-    <hyperlink ref="N149" location="SC!A1" display="SC" xr:uid="{1A712382-764E-4122-842C-18E4C1C15C55}"/>
-    <hyperlink ref="N150" location="SC!A1" display="SC" xr:uid="{E5DA2458-365F-4DEC-A5FD-D431FEAD6C7A}"/>
-    <hyperlink ref="N132:N137" location="SC!A1" display="SC" xr:uid="{1A23BD01-C554-402F-8DD0-9F9EAAD41F79}"/>
-    <hyperlink ref="I146" location="SC!A1" display="SC!A1" xr:uid="{FB1D63A9-E129-4ECF-A3EC-A22035C5490F}"/>
-    <hyperlink ref="I147" location="SC!A1" display="SC!A1" xr:uid="{2311DA73-D424-44D9-9A0B-79645D95EDE3}"/>
-    <hyperlink ref="N151" location="SC!A1" display="SC" xr:uid="{311D9EF7-53DC-4574-86B9-AFB3A04E37DF}"/>
-    <hyperlink ref="N152" location="AE!A1" display="AE" xr:uid="{AB90172E-A60F-4773-826D-88C2FC0A6E0F}"/>
-    <hyperlink ref="N134:N139" location="SC!A1" display="SC" xr:uid="{285D5173-CD5B-4BDF-B080-79FF730BF293}"/>
-    <hyperlink ref="N143" location="SC!A1" display="SC" xr:uid="{6B314DBA-DB7F-4EE1-8102-59F45F2CCBAE}"/>
-    <hyperlink ref="I143" location="SC!A1" display="SC!A1" xr:uid="{172FF343-34AE-40C5-8625-F01F134A6CE7}"/>
-    <hyperlink ref="I148" location="SC!A1" display="SC!A1" xr:uid="{8FF95C17-3AA5-4F96-A259-131E90A186DE}"/>
-    <hyperlink ref="I150" location="SC!A1" display="SC!A1" xr:uid="{C4738F97-8134-423F-8A87-9F5B6B70F9F1}"/>
-    <hyperlink ref="I156" location="CE!A1" display="CE!A1" xr:uid="{1A33317A-9350-4DC4-A713-8A6713390C8F}"/>
-    <hyperlink ref="I157" location="RE!A1" display="RE!A1" xr:uid="{8845F07D-D4E6-4376-B855-C57C8B4DB374}"/>
-    <hyperlink ref="N160" location="SC!A1" display="SC" xr:uid="{BF01B3A4-3BC4-440F-8075-E645DA4B1AC1}"/>
-    <hyperlink ref="N161" location="SC!A1" display="SC" xr:uid="{0F740229-004D-41F2-A75E-94DDB8B6CA31}"/>
-    <hyperlink ref="N162" location="RE!A1" display="RE" xr:uid="{71EC878D-03E9-4212-8E9B-C12D50180702}"/>
-    <hyperlink ref="N144:N149" location="SC!A1" display="SC" xr:uid="{66B05D55-9183-4998-951D-61B62C521537}"/>
-    <hyperlink ref="N147" location="SC!A1" display="SC" xr:uid="{B420CFF3-0D77-47B2-80BD-97DD53DCC94C}"/>
-    <hyperlink ref="N153" location="SC!A1" display="SC" xr:uid="{38A04EFA-2BAB-47FF-B8D0-B28040EBBA64}"/>
-    <hyperlink ref="I149" location="SC!A1" display="SC!A1" xr:uid="{9216BDDB-57F7-4133-83FA-F680107609FE}"/>
-    <hyperlink ref="I151" location="SC!A1" display="SC!A1" xr:uid="{6E6B1F99-1045-4AB3-A5FA-EC04C0BFD377}"/>
-    <hyperlink ref="I158" location="RE!A1" display="RE!A1" xr:uid="{ECC8A9A8-F08C-49A4-BFF0-64AB3A4D9CC8}"/>
-    <hyperlink ref="N163" location="SC!A1" display="SC" xr:uid="{94041123-5D14-41C0-B8CA-251225E99118}"/>
-    <hyperlink ref="N145:N150" location="SC!A1" display="SC" xr:uid="{83BEFF64-479A-4C63-8F7B-5320039F1253}"/>
-    <hyperlink ref="N154" location="CE!A1" display="CE" xr:uid="{0D7032C0-7440-4B23-842F-E9A3F9F6BA9A}"/>
-    <hyperlink ref="I152" location="SC!A1" display="SC!A1" xr:uid="{422A3076-0C26-4C98-9BD4-E2D676C7863B}"/>
-    <hyperlink ref="I153" location="SC!A1" display="SC!A1" xr:uid="{191002F8-5344-4D8E-96F5-A0A4AA59C2E6}"/>
-    <hyperlink ref="I154" location="AE!A1" display="AE!A1" xr:uid="{9F24F1D4-3EDB-42E1-9811-CE9D5B7914C2}"/>
-    <hyperlink ref="I162" location="SC!A1" display="SC!A1" xr:uid="{9CB764C7-DF72-4AEA-92F2-9256FF82ABB6}"/>
-    <hyperlink ref="I163" location="SC!A1" display="SC!A1" xr:uid="{5C879610-35B0-4A12-94AB-23886FE0BE54}"/>
-    <hyperlink ref="N166" location="SC!A1" display="SC" xr:uid="{6F0F0DC3-E9EA-4125-938C-216C0F830668}"/>
-    <hyperlink ref="N167" location="SC!A1" display="SC" xr:uid="{56A24A8C-6337-47F5-95AD-2F2516560F0C}"/>
-    <hyperlink ref="N168" location="SC!A1" display="SC" xr:uid="{781D5CDF-9CAA-4109-8365-8EFF15167CD3}"/>
-    <hyperlink ref="N150:N155" location="SC!A1" display="SC" xr:uid="{4900E4E1-1DFD-42F9-92DC-8E9FE7E95B4B}"/>
-    <hyperlink ref="N156" location="SC!A1" display="SC" xr:uid="{106E4F8F-82A1-49B4-8B2A-DD546B2868FF}"/>
-    <hyperlink ref="N159" location="SC!A1" display="SC" xr:uid="{25A18D84-FD02-490C-AD9A-4998918193F0}"/>
-    <hyperlink ref="N157" location="AE!A1" display="AE" xr:uid="{7F2D49BB-EFA8-485F-999B-0F2A67FBC2F9}"/>
-    <hyperlink ref="N158" location="AE!A1" display="AE" xr:uid="{84E96D22-5C81-4428-895F-36AC465AF2EA}"/>
-    <hyperlink ref="I159" location="SC!A1" display="SC!A1" xr:uid="{03BF368F-B9FF-437C-9D53-4BE8C083123B}"/>
-    <hyperlink ref="I160" location="SC!A1" display="SC!A1" xr:uid="{996D5B8B-A451-4CAA-B41F-5668F8B3E027}"/>
-    <hyperlink ref="I161" location="SC!A1" display="SC!A1" xr:uid="{D1C0D1EB-AEB4-4D33-A0F1-14C845093323}"/>
-    <hyperlink ref="I164" location="SC!A1" display="SC!A1" xr:uid="{B3533C70-92C3-46D2-BBF6-D9343BBFB87F}"/>
-    <hyperlink ref="I166" location="SC!A1" display="SC!A1" xr:uid="{942C3D11-2ECA-4F7F-984D-75EADB78D4DE}"/>
-    <hyperlink ref="I172" location="CE!A1" display="CE!A1" xr:uid="{90E847A9-D78D-43BD-B83B-F85123998EE9}"/>
-    <hyperlink ref="I173" location="RE!A1" display="RE!A1" xr:uid="{AA639E1F-249E-4B75-979A-81D5078E0569}"/>
-    <hyperlink ref="N176" location="SC!A1" display="SC" xr:uid="{25455D3E-61AC-4049-A35F-392BB696D75C}"/>
-    <hyperlink ref="N177" location="RE!A1" display="RE" xr:uid="{E299427B-5157-4736-BB25-0AC596EEC059}"/>
-    <hyperlink ref="N178" location="RE!A1" display="RE" xr:uid="{BB6DB06E-FC21-4983-9E67-F5607A454688}"/>
-    <hyperlink ref="N160:N165" location="SC!A1" display="SC" xr:uid="{2BA4BB13-2456-4631-8EA2-0157D78EB04B}"/>
-    <hyperlink ref="N169" location="SC!A1" display="SC" xr:uid="{ABED3C66-E74A-455D-A78B-D78844DA2DD7}"/>
-    <hyperlink ref="I165" location="SC!A1" display="SC!A1" xr:uid="{BE13BAC1-E10F-4BFE-9280-18DB723B5417}"/>
-    <hyperlink ref="I167" location="SC!A1" display="SC!A1" xr:uid="{754D1177-21E6-4BD0-88E4-8676A5E78723}"/>
-    <hyperlink ref="I174" location="RE!A1" display="RE!A1" xr:uid="{1E11E5F8-7AEF-4C50-807D-6C64F2632296}"/>
-    <hyperlink ref="N179" location="SC!A1" display="SC" xr:uid="{0D818959-21B9-49BD-8EAF-5835FFEBA410}"/>
-    <hyperlink ref="N161:N166" location="SC!A1" display="SC" xr:uid="{172FDE61-0EEC-437B-8D76-357697EDD4F1}"/>
-    <hyperlink ref="N164" location="SC!A1" display="SC" xr:uid="{73E3CB88-FC92-4980-BBF1-B67437B9AA6A}"/>
-    <hyperlink ref="N170" location="AE!A1" display="AE" xr:uid="{8C802D69-CF21-4C7A-9546-DD771DF60865}"/>
-    <hyperlink ref="I168" location="SC!A1" display="SC!A1" xr:uid="{30F63E5D-DD7A-42A2-8503-149EE833F92C}"/>
-    <hyperlink ref="I175" location="SC!A1" display="SC!A1" xr:uid="{029D6F95-F140-453D-9561-F086B19F1B7B}"/>
-    <hyperlink ref="N180" location="SC!A1" display="SC" xr:uid="{8FB940C1-06ED-4332-B29A-DE72EAC7E743}"/>
-    <hyperlink ref="N162:N167" location="SC!A1" display="SC" xr:uid="{958AA7B2-3774-49C0-A8FC-0E826598A974}"/>
-    <hyperlink ref="N165" location="SC!A1" display="SC" xr:uid="{7E8E535C-211E-4BB3-990E-94BB9BCFB7DE}"/>
-    <hyperlink ref="N171" location="CE!A1" display="CE" xr:uid="{8617778B-9C70-46EB-B1B7-9888D62B3597}"/>
-    <hyperlink ref="I169" location="SC!A1" display="SC!A1" xr:uid="{6FBCE9FB-2509-490E-8B36-572C5B8DB8FD}"/>
-    <hyperlink ref="I170" location="AE!A1" display="AE!A1" xr:uid="{576CF1E7-8549-4B99-AF72-B286AA2371A2}"/>
-    <hyperlink ref="I178" location="SC!A1" display="SC!A1" xr:uid="{D0ADF097-728C-4778-94D7-60D031072162}"/>
-    <hyperlink ref="I179" location="SC!A1" display="SC!A1" xr:uid="{AC583000-D467-404F-BA6A-698A03ACC9CE}"/>
-    <hyperlink ref="N182" location="SC!A1" display="SC" xr:uid="{E1FBDB5B-B81E-4DBB-8CB0-D88E5F82693A}"/>
-    <hyperlink ref="N183" location="SC!A1" display="SC" xr:uid="{EFBC9873-11D6-4C15-A68D-E3F7294AEB61}"/>
-    <hyperlink ref="N184" location="AE!A1" display="AE" xr:uid="{1E3C5B3C-D9D8-4594-BC58-9F8BA0FC93AE}"/>
-    <hyperlink ref="N166:N171" location="SC!A1" display="SC" xr:uid="{68268FE8-E28D-46F9-AB93-31ED9AE692BE}"/>
-    <hyperlink ref="N172" location="SC!A1" display="SC" xr:uid="{F22E9F0D-B193-416A-84BF-1D61D9E8AB27}"/>
-    <hyperlink ref="N175" location="SC!A1" display="SC" xr:uid="{C079AD68-069C-4852-BFA4-67365EC5672E}"/>
-    <hyperlink ref="N173" location="AE!A1" display="AE" xr:uid="{F9392CB2-E57D-4527-8638-17502980A2CA}"/>
-    <hyperlink ref="N174" location="AE!A1" display="AE" xr:uid="{9FAE2560-8451-4B5E-A921-EE080355DCC2}"/>
-    <hyperlink ref="I176" location="SC!A1" display="SC!A1" xr:uid="{7C6585D4-E185-433A-97A9-3C100B971A6F}"/>
-    <hyperlink ref="I177" location="SC!A1" display="SC!A1" xr:uid="{4E6F3741-4F84-4842-A250-43A74CE24FCE}"/>
-    <hyperlink ref="I180" location="SC!A1" display="SC!A1" xr:uid="{F5A9E2D5-9A77-4C7A-83BE-24420290AF2E}"/>
-    <hyperlink ref="I182" location="SC!A1" display="SC!A1" xr:uid="{A586A2B3-7E6D-41D1-A0EC-99A49D00AE2C}"/>
-    <hyperlink ref="I188" location="CE!A1" display="CE!A1" xr:uid="{78AB49F7-8A1A-43FA-A528-3375B1FB1AF1}"/>
-    <hyperlink ref="I189" location="RE!A1" display="RE!A1" xr:uid="{A8CA8328-B927-47CC-9B6E-7B7A01816551}"/>
-    <hyperlink ref="N192" location="SC!A1" display="SC" xr:uid="{308C0216-1366-478D-9F50-436B93D01122}"/>
-    <hyperlink ref="N193" location="SC!A1" display="SC" xr:uid="{5DE2A861-87E1-4561-89FD-27067BF56ADD}"/>
-    <hyperlink ref="N194" location="RE!A1" display="RE" xr:uid="{10097251-6DE0-4EE1-880C-23B16C22B277}"/>
-    <hyperlink ref="N176:N181" location="SC!A1" display="SC" xr:uid="{3049DD10-1851-438D-AD81-85DBFCF69735}"/>
-    <hyperlink ref="N185" location="SC!A1" display="SC" xr:uid="{039E4502-C5F2-4EE2-B69C-502380622175}"/>
-    <hyperlink ref="I181" location="SC!A1" display="SC!A1" xr:uid="{748585F2-77EB-4DBA-BE36-65964EE87B0E}"/>
-    <hyperlink ref="I183" location="SC!A1" display="SC!A1" xr:uid="{147B75B7-A547-4C72-9465-4621049E23E5}"/>
-    <hyperlink ref="I190" location="RE!A1" display="RE!A1" xr:uid="{F1CE491C-17B4-4811-A22B-00F79C9FEF3B}"/>
-    <hyperlink ref="N195" location="SC!A1" display="SC" xr:uid="{8721B5FB-B2D4-419E-98EB-256978D7E3DD}"/>
-    <hyperlink ref="N177:N182" location="SC!A1" display="SC" xr:uid="{ABE55AD1-3611-41FA-B6A4-F8E55778F144}"/>
-    <hyperlink ref="N186" location="CE!A1" display="CE" xr:uid="{69C8CFA4-86E9-408D-AFBC-7A6660D3D813}"/>
-    <hyperlink ref="I184" location="SC!A1" display="SC!A1" xr:uid="{3C899473-6CF3-43A1-A325-7FD5254E1311}"/>
-    <hyperlink ref="I185" location="SC!A1" display="SC!A1" xr:uid="{F310013F-3D4B-4CEE-B553-F420D1874528}"/>
-    <hyperlink ref="I194" location="SC!A1" display="SC!A1" xr:uid="{FFEFA734-BE02-4548-9664-54A722AF4EF7}"/>
-    <hyperlink ref="I195" location="SC!A1" display="SC!A1" xr:uid="{1710478C-D7F6-4A96-BABC-D40CD5A4FF37}"/>
-    <hyperlink ref="N181" location="SC!A1" display="SC" xr:uid="{AA28EC25-F2E7-47D5-BAE3-E7CB56E9967C}"/>
-    <hyperlink ref="N198" location="SC!A1" display="SC" xr:uid="{2ECA08C4-F7A7-46CE-86EF-26B102C7DFDF}"/>
-    <hyperlink ref="N199" location="SC!A1" display="SC" xr:uid="{FF6B9045-FFAE-4DEB-9670-56055DD605E0}"/>
-    <hyperlink ref="N200" location="SC!A1" display="SC" xr:uid="{7F0137EE-0C38-4A30-8F61-7A854FA900AF}"/>
-    <hyperlink ref="N182:N187" location="SC!A1" display="SC" xr:uid="{F2F7B7D4-8D72-41CF-8EE2-D478004825CF}"/>
-    <hyperlink ref="N188" location="SC!A1" display="SC" xr:uid="{7E7103A1-4273-4AD2-AE06-44BB9C2BE6B2}"/>
-    <hyperlink ref="N191" location="SC!A1" display="SC" xr:uid="{A07695B2-C683-44C8-8288-0004D1FFF544}"/>
-    <hyperlink ref="N189" location="AE!A1" display="AE" xr:uid="{1BC430FF-E5F7-43A5-AEB1-985F67E9DFE7}"/>
-    <hyperlink ref="N190" location="AE!A1" display="AE" xr:uid="{79855B4A-7A78-4266-A950-DA0885F04B35}"/>
-    <hyperlink ref="I191" location="SC!A1" display="SC!A1" xr:uid="{6B30536A-0C4C-426D-AB2D-8F0CD74A72CC}"/>
-    <hyperlink ref="I192" location="SC!A1" display="SC!A1" xr:uid="{F63B94FB-9388-4EB8-9AE8-E572DEA75A2F}"/>
-    <hyperlink ref="I193" location="SC!A1" display="SC!A1" xr:uid="{9236D2E2-29A9-4899-B365-F4EAFA25F115}"/>
-    <hyperlink ref="I196" location="SC!A1" display="SC!A1" xr:uid="{A9559F6D-F5CD-486B-8F7F-A303335DCF08}"/>
-    <hyperlink ref="I198" location="AE!A1" display="AE!A1" xr:uid="{E389905A-9312-4AD7-B5A0-11E7285BECA3}"/>
-    <hyperlink ref="I204" location="AE!A1" display="AE!A1" xr:uid="{C4DA0F9A-C3B0-4D87-A29E-D8F18E0CC324}"/>
-    <hyperlink ref="I205" location="SC!A1" display="SC!A1" xr:uid="{52870DB8-945E-4FAE-984A-2E1653201FC6}"/>
-    <hyperlink ref="N208" location="SC!A1" display="SC" xr:uid="{8753B2E8-FA82-4689-B416-C49AAF915C51}"/>
-    <hyperlink ref="N209" location="SC!A1" display="SC" xr:uid="{2803F427-6792-4C72-A884-A9C17FDAC8E7}"/>
-    <hyperlink ref="N210" location="RE!A1" display="RE" xr:uid="{8236795D-3059-4FDF-8B26-02751024F8CB}"/>
-    <hyperlink ref="N192:N197" location="SC!A1" display="SC" xr:uid="{29000766-8EC4-4FE9-915A-F64517967003}"/>
-    <hyperlink ref="N201" location="AE!A1" display="AE" xr:uid="{179B9B8D-E047-4FE8-B666-82ADC1DBF2B4}"/>
-    <hyperlink ref="I197" location="SC!A1" display="SC!A1" xr:uid="{B2B0792F-624A-42B3-9038-1CE453F6A310}"/>
-    <hyperlink ref="I199" location="SC!A1" display="SC!A1" xr:uid="{79899498-F728-4DEC-9AFE-617D36333640}"/>
-    <hyperlink ref="I206" location="SC!A1" display="SC!A1" xr:uid="{438C87EF-468E-4E3B-80E9-8AFBEFD370CB}"/>
-    <hyperlink ref="N211" location="SC!A1" display="SC" xr:uid="{909C2401-406A-42CD-B274-71486B60E619}"/>
-    <hyperlink ref="N193:N198" location="SC!A1" display="SC" xr:uid="{B29F7847-5058-4784-9E5C-8A796C98E2BE}"/>
-    <hyperlink ref="N196" location="SC!A1" display="SC" xr:uid="{6E218A04-ACC6-4554-B131-68F11E937D7C}"/>
-    <hyperlink ref="N202" location="AE!A1" display="AE" xr:uid="{159B7B92-01E6-47DB-A65A-9913D332E4A5}"/>
-    <hyperlink ref="I200" location="SC!A1" display="SC!A1" xr:uid="{FE839DA9-F37B-4117-8C79-B5EEE49B655A}"/>
-    <hyperlink ref="I207" location="SC!A1" display="SC!A1" xr:uid="{035E2CE4-ED73-448C-B9EA-0B983AA01062}"/>
-    <hyperlink ref="N212" location="SC!A1" display="SC" xr:uid="{808AE38F-8052-4DD9-905D-B7C3A8765518}"/>
-    <hyperlink ref="N194:N199" location="SC!A1" display="SC" xr:uid="{98C64EC5-865F-42AD-BE01-EB20761DE9AE}"/>
-    <hyperlink ref="N197" location="SC!A1" display="SC" xr:uid="{B54F6E86-402E-46B9-AAA7-52946866763E}"/>
-    <hyperlink ref="N203" location="SC!A1" display="SC" xr:uid="{2AD97E2D-9E7C-4621-833E-BD41AFC1B750}"/>
-    <hyperlink ref="I201" location="SC!A1" display="SC!A1" xr:uid="{05A27030-EC9D-4685-8D32-D9970D7B2951}"/>
-    <hyperlink ref="I202" location="SC!A1" display="SC!A1" xr:uid="{30940271-8F5C-4A60-9B43-90192DEB5A41}"/>
-    <hyperlink ref="I203" location="SC!A1" display="SC!A1" xr:uid="{629C7FCE-0A8E-4D5A-9E6A-8B92922C815C}"/>
-    <hyperlink ref="I212" location="SC!A1" display="SC!A1" xr:uid="{D6531378-3ADB-4E75-A8D2-E090B6C6F8E0}"/>
-    <hyperlink ref="I213" location="SC!A1" display="SC!A1" xr:uid="{B24F8967-C09D-4F0E-9D13-24D4FB9C0DC7}"/>
-    <hyperlink ref="N216" location="AE!A1" display="AE" xr:uid="{39ADDA20-6435-451E-BC13-859E38107156}"/>
-    <hyperlink ref="N217" location="AE!A1" display="AE" xr:uid="{6107402C-5FBC-4AFD-B401-F935888BFAEE}"/>
-    <hyperlink ref="N218" location="SC!A1" display="SC" xr:uid="{EC8A37D8-8223-4CE7-BCC4-622FD2D5FAB3}"/>
-    <hyperlink ref="N200:N205" location="SC!A1" display="SC" xr:uid="{EAF1D838-772C-4A6D-8B0A-A49B0D3DB7D1}"/>
-    <hyperlink ref="N206" location="SC!A1" display="SC" xr:uid="{1699BC08-7E37-49B3-975A-745AA75B36A5}"/>
-    <hyperlink ref="N207" location="AE!A1" display="AE" xr:uid="{4FE1F724-110F-4270-B2B5-70637517E98F}"/>
-    <hyperlink ref="I208" location="SC!A1" display="SC!A1" xr:uid="{4A022ECB-976F-493C-84F6-7483243205FD}"/>
-    <hyperlink ref="I209" location="SC!A1" display="SC!A1" xr:uid="{B829CA89-E67E-4663-AF62-2AD4D6393FD2}"/>
-    <hyperlink ref="I210" location="SC!A1" display="SC!A1" xr:uid="{E55FEC92-C5DF-48B4-BE78-C43F9793F78E}"/>
-    <hyperlink ref="I218" location="CE!A1" display="CE!A1" xr:uid="{76E20186-E4B6-47E8-A86E-07E24FE805B9}"/>
-    <hyperlink ref="I219" location="RE!A1" display="RE!A1" xr:uid="{A3585F56-306B-4EC4-ABB3-E15A7A73B90F}"/>
-    <hyperlink ref="N205" location="SC!A1" display="SC" xr:uid="{47D47C5B-EDB6-4ED4-8FEE-5750F434F766}"/>
-    <hyperlink ref="N221" location="RE!A1" display="RE" xr:uid="{26E9025F-5D9A-4F6E-9C74-0431EF3FC2FC}"/>
-    <hyperlink ref="N222" location="SC!A1" display="SC" xr:uid="{44D3E3B4-D17D-4F58-83CD-74672495D6EE}"/>
-    <hyperlink ref="N223" location="RE!A1" display="RE" xr:uid="{944CC584-D41E-415F-9F76-1AAA0260B58A}"/>
-    <hyperlink ref="N206:N211" location="SC!A1" display="SC" xr:uid="{3B3B3FB1-1DCD-4CAB-ADB8-0C9F7232774D}"/>
-    <hyperlink ref="N215" location="SC!A1" display="SC" xr:uid="{D28E0160-A65F-4130-9421-1507CCD92310}"/>
-    <hyperlink ref="N213" location="AE!A1" display="AE" xr:uid="{ED547ACB-E1B9-4963-9257-8BFFEFD14AA2}"/>
-    <hyperlink ref="N214" location="AE!A1" display="AE" xr:uid="{15802B6F-560C-4947-ADA6-33595D667531}"/>
-    <hyperlink ref="I211" location="SC!A1" display="SC!A1" xr:uid="{80279D3A-EED3-4EEA-9FF7-F990EC627AAA}"/>
-    <hyperlink ref="I215" location="SC!A1" display="SC!A1" xr:uid="{F77A7291-2893-4FE5-ACC2-A405336B81D6}"/>
-    <hyperlink ref="I221" location="RE!A1" display="RE!A1" xr:uid="{21CD6632-C12E-43C4-B69A-F5DD56483465}"/>
-    <hyperlink ref="N224" location="SC!A1" display="SC" xr:uid="{5DF9F6E3-5E73-46BC-892C-582FD005927F}"/>
-    <hyperlink ref="N225" location="RE!A1" display="RE" xr:uid="{03ADA734-EE6C-4287-A7F3-3C22129A9B08}"/>
-    <hyperlink ref="N226" location="SC!A1" display="SC" xr:uid="{B1CCAE35-A251-4EA9-B906-6B8633F7F737}"/>
-    <hyperlink ref="N209:N214" location="SC!A1" display="SC" xr:uid="{39CB0E9E-7B75-450A-80FE-39C23684C33D}"/>
-    <hyperlink ref="I214" location="SC!A1" display="SC!A1" xr:uid="{8A8F5925-C398-4B1D-8113-E0CC771C8473}"/>
-    <hyperlink ref="I216" location="AE!A1" display="AE!A1" xr:uid="{B18C773B-A819-4358-ACC3-C9709FED5502}"/>
-    <hyperlink ref="I223" location="SC!A1" display="SC!A1" xr:uid="{46305BA4-8274-48F2-BBFF-A6A5B791B02C}"/>
-    <hyperlink ref="I224" location="SC!A1" display="SC!A1" xr:uid="{3E97EB9F-CF6C-4DA3-BEB9-52A37E1DEE59}"/>
-    <hyperlink ref="N227" location="RE!A1" display="RE" xr:uid="{D1B35183-BF21-44C4-9A88-BA250C2D1044}"/>
-    <hyperlink ref="N228" location="SC!A1" display="SC" xr:uid="{9279DAF4-AE55-4A15-8704-D7DEAA7FFBF4}"/>
-    <hyperlink ref="N229" location="SC!A1" display="SC" xr:uid="{B62E9393-14E4-489E-9F32-28AB97C35C50}"/>
-    <hyperlink ref="N212:N217" location="SC!A1" display="SC" xr:uid="{ADF5EEA3-48D6-4710-869B-979502E72FCF}"/>
-    <hyperlink ref="N219" location="AE!A1" display="AE" xr:uid="{A613DC09-A0D8-4B69-9530-436B0E5EE72D}"/>
-    <hyperlink ref="N220" location="AE!A1" display="AE" xr:uid="{6839F5D4-EF5B-442D-B01C-FF2E82DA23CF}"/>
-    <hyperlink ref="I222" location="SC!A1" display="SC!A1" xr:uid="{726C561D-E7AB-44B4-95B3-E83F8D2D0F2B}"/>
-    <hyperlink ref="I225" location="SC!A1" display="SC!A1" xr:uid="{633BE0FA-78BE-4AB6-A1D8-6D6F1FDE162B}"/>
-    <hyperlink ref="I226" location="SC!A1" display="SC!A1" xr:uid="{15F64AC7-878B-4F04-BA49-7F334B94F044}"/>
-    <hyperlink ref="I227" location="SC!A1" display="SC!A1" xr:uid="{73C69F1A-85B5-40E0-B4A7-30093B4D4374}"/>
-    <hyperlink ref="I229" location="AE!A1" display="AE!A1" xr:uid="{3C0FB6EF-A693-44A8-AC64-6909617F828E}"/>
-    <hyperlink ref="I235" location="SC!A1" display="SC!A1" xr:uid="{4ED5EECD-D25A-4F40-8AB7-C0F4296BA84B}"/>
-    <hyperlink ref="I236" location="SC!A1" display="SC!A1" xr:uid="{BE9CB7E4-43FA-4501-B528-E0D61D232A1A}"/>
-    <hyperlink ref="N239" location="RE!A1" display="RE" xr:uid="{101FEF7F-4F32-43B8-96E5-3645BDFD4786}"/>
-    <hyperlink ref="N240" location="RE!A1" display="RE" xr:uid="{E1AE7184-3E5C-427D-A59B-7148C44FA687}"/>
-    <hyperlink ref="N223:N228" location="SC!A1" display="SC" xr:uid="{0A918722-85E4-4C12-A6C5-F4A2E8E6002D}"/>
-    <hyperlink ref="N232" location="AE!A1" display="AE" xr:uid="{69015DAA-F6A0-4022-A9C1-E4C3CDF2E6FC}"/>
-    <hyperlink ref="N230" location="AE!A1" display="AE" xr:uid="{5C12D3BF-10CB-471F-BF7A-8023861BD48E}"/>
-    <hyperlink ref="N231" location="SC!A1" display="SC" xr:uid="{FE9F4E27-6912-4F16-8FCC-38D04AC1D960}"/>
-    <hyperlink ref="I228" location="SC!A1" display="SC!A1" xr:uid="{C694B438-A99D-45BA-8668-7F734BA9D62E}"/>
-    <hyperlink ref="I231" location="CE!A1" display="CE!A1" xr:uid="{9B34F849-33EC-427A-8D52-F91F8D627557}"/>
-    <hyperlink ref="I237" location="SC!A1" display="SC!A1" xr:uid="{9480E0AB-E02D-49A5-8D92-7CE96306B491}"/>
-    <hyperlink ref="I238" location="SC!A1" display="SC!A1" xr:uid="{E426F211-200C-4662-BBDB-B3E2E8559026}"/>
-    <hyperlink ref="N225:N230" location="SC!A1" display="SC" xr:uid="{A4AE0195-0748-49CA-BA83-60DF66D7AEC6}"/>
-    <hyperlink ref="N234" location="SC!A1" display="SC" xr:uid="{8237B9A4-E955-4DE6-8EB8-803C60E5101F}"/>
-    <hyperlink ref="N233" location="AE!A1" display="AE" xr:uid="{D145410E-87C8-415D-BDDA-17CB4F82A046}"/>
-    <hyperlink ref="I234" location="SC!A1" display="SC!A1" xr:uid="{CCAE8155-6AB1-45ED-8158-50CAF0D12A77}"/>
-    <hyperlink ref="I239" location="AE!A1" display="AE!A1" xr:uid="{8DEB6192-CF7C-4513-B01A-D20BEEE9E910}"/>
-    <hyperlink ref="I243" location="RE!A1" display="RE!A1" xr:uid="{BC26B786-A9DB-4934-A0AF-67172E71856D}"/>
-    <hyperlink ref="I244" location="RE!A1" display="RE!A1" xr:uid="{F33D4E58-B0E4-4789-A5FE-3AAABF2AC8B0}"/>
-    <hyperlink ref="N247" location="RE!A1" display="RE" xr:uid="{32336C2B-C00F-4BD8-9FAC-C8E1DC09D5E9}"/>
-    <hyperlink ref="N248" location="RE!A1" display="RE" xr:uid="{3D1241B2-6011-4215-846D-C6319BF8B532}"/>
-    <hyperlink ref="N249" location="RE!A1" display="RE" xr:uid="{E92AF947-746F-43AB-A6FA-722C14664660}"/>
-    <hyperlink ref="N235:N240" location="SC!A1" display="SC" xr:uid="{55E325A1-1A10-420E-8D5E-093AF71CD4C1}"/>
-    <hyperlink ref="N238" location="SC!A1" display="SC" xr:uid="{198BB2EA-0C40-40A2-89B7-C8752B2E8525}"/>
-    <hyperlink ref="I299" location="SC!A1" display="SC!A1" xr:uid="{2A2CF76F-71CE-4523-ADD4-9B7511572A35}"/>
-    <hyperlink ref="I300" location="AE!A1" display="AE!A1" xr:uid="{36885424-E0A7-475D-B167-FDA75EE01DC2}"/>
-    <hyperlink ref="I302" location="AE!A1" display="AE!A1" xr:uid="{8CAAED43-94CC-49B3-AFAB-65EFE65464A3}"/>
-    <hyperlink ref="I308" location="RE!A1" display="RE!A1" xr:uid="{FFDACA7E-B33F-4653-9F74-0FBDC2DAE97E}"/>
-    <hyperlink ref="I309" location="RE!A1" display="RE!A1" xr:uid="{EFC3884D-EF9C-40F9-A73E-6145A16B4E01}"/>
-    <hyperlink ref="N299" location="SC!A1" display="SC" xr:uid="{E14940FE-5FCF-44AA-8D44-5859E1F1BB45}"/>
-    <hyperlink ref="N532" location="RE!A1" display="RE" xr:uid="{A90C7ACA-A1B1-432E-B9FB-91D8DD1A7D83}"/>
-    <hyperlink ref="N312" location="RE!A1" display="RE" xr:uid="{C54E5A54-5FF0-4845-81FE-F83AB7A7D6EE}"/>
-    <hyperlink ref="N300:N301" location="SC!A1" display="SC" xr:uid="{840F82EE-84DC-4F44-9268-74287D8A9A0B}"/>
-    <hyperlink ref="N302" location="SC!A1" display="SC" xr:uid="{8AC3E057-3294-464B-850D-8B622F0C6137}"/>
-    <hyperlink ref="N305" location="AE!A1" display="AE" xr:uid="{4E873342-7B74-4E0D-8D37-DD10961E9EAB}"/>
-    <hyperlink ref="N303" location="AE!A1" display="AE" xr:uid="{228BE4CD-D01C-4191-988D-BF6D052D48C2}"/>
-    <hyperlink ref="N304" location="SC!A1" display="SC" xr:uid="{7A2A23B7-56B6-4391-AD01-F4AB7C4C0E62}"/>
-    <hyperlink ref="I301" location="SC!A1" display="SC!A1" xr:uid="{92A84750-3E8B-437C-8C49-815C58EA70E4}"/>
-    <hyperlink ref="I304" location="RE!A1" display="RE!A1" xr:uid="{2E8F1CE8-5BF9-41F2-9FDA-21C124DC1D46}"/>
-    <hyperlink ref="I310" location="RE!A1" display="RE!A1" xr:uid="{5ACD07C1-DEED-4656-9746-763B2EEAA1CA}"/>
-    <hyperlink ref="N313" location="RE!A1" display="RE" xr:uid="{7BA923BB-5F23-49F9-8C65-4E022CCFB367}"/>
-    <hyperlink ref="N301:N303" location="SC!A1" display="SC" xr:uid="{6E09B929-95FF-4C71-B555-05A73ADD2B8F}"/>
-    <hyperlink ref="N301" location="CE!A1" display="CE" xr:uid="{30308A3D-052A-47DF-9E15-A647F8F4427C}"/>
-    <hyperlink ref="N307" location="CE!A1" display="CE" xr:uid="{1E2B95B9-0D07-46B4-90B0-23F94605065B}"/>
-    <hyperlink ref="N306" location="AE!A1" display="AE" xr:uid="{4F5B276E-F7A8-46B8-9539-93B67393A92F}"/>
-    <hyperlink ref="I291" location="SC!A1" display="SC!A1" xr:uid="{2148388B-4231-4866-BEE8-FB576FBF577E}"/>
-    <hyperlink ref="I292" location="SC!A1" display="SC!A1" xr:uid="{EFB36E16-0674-4789-8812-E1E26C9BCB5D}"/>
-    <hyperlink ref="I297" location="SC!A1" display="SC!A1" xr:uid="{61B1DC82-4CF3-4A69-A2FF-E06F79732DA9}"/>
-    <hyperlink ref="I298" location="SC!A1" display="SC!A1" xr:uid="{7BEF901A-B366-4A3A-8829-473AA598CE2C}"/>
-    <hyperlink ref="I305" location="RE!A1" display="RE!A1" xr:uid="{9E890CB3-181E-42EB-B39D-3052F9A385CB}"/>
-    <hyperlink ref="N308" location="RE!A1" display="RE" xr:uid="{67D09BE0-3456-4A47-96F5-6467B3EA46D3}"/>
-    <hyperlink ref="N309" location="RE!A1" display="RE" xr:uid="{E4E00ADA-89FC-48C1-9290-895EBB57F0AB}"/>
-    <hyperlink ref="N310" location="RE!A1" display="RE" xr:uid="{DC5CFD2C-9623-434D-9FE6-3FD34F92F97E}"/>
-    <hyperlink ref="N292:N300" location="SC!A1" display="SC" xr:uid="{2C09D4F7-71C2-4579-92A3-0D258E7E1F08}"/>
-    <hyperlink ref="N53:N58" location="SC!A1" display="SC" xr:uid="{469E8262-7D88-4B63-B5EC-9C6DFE18A5B8}"/>
-    <hyperlink ref="N52:N57" location="SC!A1" display="SC" xr:uid="{764ADB42-7E3C-459D-BF8D-2157A3436BE3}"/>
-    <hyperlink ref="N50:N55" location="SC!A1" display="SC" xr:uid="{904BC71B-6958-4892-829D-38FAE06297ED}"/>
-    <hyperlink ref="N49:N54" location="SC!A1" display="SC" xr:uid="{F47FEC58-EF0F-4A25-A84F-D6382940F9CC}"/>
-    <hyperlink ref="N47:N52" location="SC!A1" display="SC" xr:uid="{3BE9B0B5-BE59-41E8-9428-927E3BCA49A0}"/>
-    <hyperlink ref="N46:N51" location="SC!A1" display="SC" xr:uid="{CC1E187F-6232-452F-A0A4-DA510A8FC8AB}"/>
-    <hyperlink ref="N44:N49" location="SC!A1" display="SC" xr:uid="{81F2BBAE-FD79-43B4-A632-08ECC1B0D0BA}"/>
-    <hyperlink ref="N43:N48" location="SC!A1" display="SC" xr:uid="{E5923857-9557-44AA-B5CD-812B340CAB9B}"/>
-    <hyperlink ref="N42:N46" location="SC!A1" display="SC" xr:uid="{B83F3552-1BC2-4C71-A43F-CBE5963A6A86}"/>
-    <hyperlink ref="N41:N45" location="SC!A1" display="SC" xr:uid="{DA8FC7CE-4E39-470D-8F97-E7BAC39F83F5}"/>
-    <hyperlink ref="N58" location="SC!A1" display="SC" xr:uid="{56A148A8-EB3C-416E-9B52-09ACB7829953}"/>
-    <hyperlink ref="N57" location="AE!A1" display="AE" xr:uid="{F41900DA-2A63-4186-BB5D-102CA8CED99E}"/>
-    <hyperlink ref="N39:N43" location="SC!A1" display="SC" xr:uid="{49D83FB1-6C7B-45CE-A3BC-12CC4D81214C}"/>
-    <hyperlink ref="N56" location="SC!A1" display="SC" xr:uid="{CEF05C6E-84ED-41B7-9DF9-D031BF0705EE}"/>
-    <hyperlink ref="N38:N42" location="SC!A1" display="SC" xr:uid="{EF121C1B-7457-409D-89F9-B55446A3A885}"/>
-    <hyperlink ref="N55" location="SC!A1" display="SC" xr:uid="{C22B0F9C-E50A-423B-B51A-7679DB28BC52}"/>
-    <hyperlink ref="N54" location="SC!A1" display="SC" xr:uid="{2710978C-5410-4980-A154-B845FC4225ED}"/>
-    <hyperlink ref="N36:N41" location="SC!A1" display="SC" xr:uid="{CB13A3E9-CA6C-403C-818F-9F931F9A1F1D}"/>
-    <hyperlink ref="N53" location="SC!A1" display="SC" xr:uid="{1DC53BEE-1E91-455C-AFFB-CF56925381D9}"/>
-    <hyperlink ref="N35:N40" location="SC!A1" display="SC" xr:uid="{30AEC6E7-2694-4949-BBCC-CD2AC6E81BE4}"/>
-    <hyperlink ref="N52" location="SC!A1" display="SC" xr:uid="{2E6B148B-9D9A-44D9-AFC4-F7F570FAE0E6}"/>
-    <hyperlink ref="N51" location="SC!A1" display="SC" xr:uid="{DB4E9CCE-C4A4-4838-AB99-B5D6C8FA4C9B}"/>
-    <hyperlink ref="N33:N38" location="SC!A1" display="SC" xr:uid="{B865897A-203C-4959-86CA-71E8A1173522}"/>
-    <hyperlink ref="N50" location="SC!A1" display="SC" xr:uid="{0B325584-192D-4B68-B870-BE742740792F}"/>
-    <hyperlink ref="N33:N37" location="SC!A1" display="SC" xr:uid="{08D46D21-22EF-49CE-B697-4A3C3427E51C}"/>
-    <hyperlink ref="N49" location="SC!A1" display="SC" xr:uid="{F18ED71B-6742-4CD1-9A5B-1FCE793B8787}"/>
-    <hyperlink ref="N48" location="SC!A1" display="SC" xr:uid="{78FF8EAE-FAD2-40B1-A676-7A363EF06EC6}"/>
-    <hyperlink ref="N47" location="SC!A1" display="SC" xr:uid="{58F3AC7F-EAA6-4039-B0FB-A3D48A5DCFDE}"/>
-    <hyperlink ref="N46" location="SC!A1" display="SC" xr:uid="{9CAE7468-5579-497B-A97B-E1B1FCCB0A62}"/>
-    <hyperlink ref="N45" location="SC!A1" display="SC" xr:uid="{A056E7E1-5731-473F-B4E1-28FD29551D61}"/>
-    <hyperlink ref="N44" location="SC!A1" display="SC" xr:uid="{BBF80776-4EF3-47AA-8822-9C0FFFCF3C19}"/>
-    <hyperlink ref="N43" location="SC!A1" display="SC" xr:uid="{F82C10D3-3395-43CE-857F-10DE605627E1}"/>
-    <hyperlink ref="N42" location="SC!A1" display="SC" xr:uid="{CD833979-8E38-44DD-9B4E-B3E163E3D7D6}"/>
-    <hyperlink ref="N41" location="SC!A1" display="SC" xr:uid="{727E66AE-160F-4CB3-8043-49F7848BD653}"/>
-    <hyperlink ref="N40" location="SC!A1" display="SC" xr:uid="{E03DBB8F-79A8-4B59-BF59-5A8D0317B26B}"/>
-    <hyperlink ref="N39" location="SC!A1" display="SC" xr:uid="{C1030103-E114-4B7E-8D52-736D6C73D165}"/>
-    <hyperlink ref="N38" location="SC!A1" display="SC" xr:uid="{AA955B7C-41DB-41A6-BCF5-BE8D5A1EC8B1}"/>
-    <hyperlink ref="N37" location="SC!A1" display="SC" xr:uid="{949B88C7-5304-4202-92B8-5624EB9AB638}"/>
-    <hyperlink ref="N36" location="SC!A1" display="SC" xr:uid="{2620164D-88A6-493F-82D0-82C60D83E521}"/>
-    <hyperlink ref="N35" location="SC!A1" display="SC" xr:uid="{A9E63502-61E7-431C-A0E0-9E23AFFC31DD}"/>
-    <hyperlink ref="N34" location="SC!A1" display="SC" xr:uid="{0E9AA225-C2A9-43C1-9C5E-934C5658FC2F}"/>
-    <hyperlink ref="N33" location="SC!A1" display="SC" xr:uid="{04694F74-C82E-4642-8DEE-11304626517F}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>